<commit_message>
Update GPU prices and charts - 2026-09-13 14:44:01
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2845" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2864" uniqueCount="100">
   <si>
     <t>Date</t>
   </si>
@@ -322,6 +322,9 @@
   </si>
   <si>
     <t>2026-09-12</t>
+  </si>
+  <si>
+    <t>2026-09-13</t>
   </si>
 </sst>
 </file>
@@ -1228,7 +1231,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C96"/>
+  <dimension ref="A1:C97"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2292,6 +2295,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="97" spans="1:3" ht="16" customHeight="1">
+      <c r="A97" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C97" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2300,7 +2314,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C96"/>
+  <dimension ref="A1:C97"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3364,6 +3378,17 @@
         <v>2.39</v>
       </c>
     </row>
+    <row r="97" spans="1:3" ht="16" customHeight="1">
+      <c r="A97" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B97" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C97" s="3">
+        <v>2.39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3372,7 +3397,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C96"/>
+  <dimension ref="A1:C97"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4436,6 +4461,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="97" spans="1:3" ht="16" customHeight="1">
+      <c r="A97" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B97" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C97" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4444,7 +4480,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C96"/>
+  <dimension ref="A1:C97"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5508,6 +5544,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="97" spans="1:3" ht="16" customHeight="1">
+      <c r="A97" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C97" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5516,7 +5563,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C96"/>
+  <dimension ref="A1:C97"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6580,6 +6627,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="97" spans="1:3" ht="16" customHeight="1">
+      <c r="A97" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C97" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6588,7 +6646,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C96"/>
+  <dimension ref="A1:C97"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7652,6 +7710,17 @@
         <v>6.79</v>
       </c>
     </row>
+    <row r="97" spans="1:3" ht="16" customHeight="1">
+      <c r="A97" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B97" s="3">
+        <v>3.75</v>
+      </c>
+      <c r="C97" s="3">
+        <v>6.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7660,7 +7729,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C96"/>
+  <dimension ref="A1:C97"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8724,6 +8793,17 @@
         <v>4.1973</v>
       </c>
     </row>
+    <row r="97" spans="1:3" ht="16" customHeight="1">
+      <c r="A97" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B97" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C97" s="3">
+        <v>4.6933</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8732,7 +8812,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C96"/>
+  <dimension ref="A1:C97"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9796,6 +9876,17 @@
         <v>3.6842</v>
       </c>
     </row>
+    <row r="97" spans="1:3" ht="16" customHeight="1">
+      <c r="A97" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B97" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C97" s="3">
+        <v>3.6842</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9804,7 +9895,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C96"/>
+  <dimension ref="A1:C97"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10868,6 +10959,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="97" spans="1:3" ht="16" customHeight="1">
+      <c r="A97" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B97" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C97" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10876,7 +10978,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C96"/>
+  <dimension ref="A1:C97"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11940,6 +12042,17 @@
         <v>3.49</v>
       </c>
     </row>
+    <row r="97" spans="1:3" ht="16" customHeight="1">
+      <c r="A97" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B97" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C97" s="3">
+        <v>2.8533</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11948,7 +12061,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C96"/>
+  <dimension ref="A1:C97"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13012,6 +13125,17 @@
         <v>3.1467</v>
       </c>
     </row>
+    <row r="97" spans="1:3" ht="16" customHeight="1">
+      <c r="A97" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B97" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C97" s="3">
+        <v>2.8667</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13020,7 +13144,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C96"/>
+  <dimension ref="A1:C97"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14084,6 +14208,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="97" spans="1:3" ht="16" customHeight="1">
+      <c r="A97" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C97" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-14 16:39:46
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2864" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2884" uniqueCount="101">
   <si>
     <t>Date</t>
   </si>
@@ -325,6 +325,9 @@
   </si>
   <si>
     <t>2026-09-13</t>
+  </si>
+  <si>
+    <t>2026-09-14</t>
   </si>
 </sst>
 </file>
@@ -1231,7 +1234,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C97"/>
+  <dimension ref="A1:C98"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2306,6 +2309,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="98" spans="1:3" ht="16" customHeight="1">
+      <c r="A98" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B98" s="3">
+        <v>7.651</v>
+      </c>
+      <c r="C98" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2314,7 +2328,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C97"/>
+  <dimension ref="A1:C98"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3389,6 +3403,17 @@
         <v>2.39</v>
       </c>
     </row>
+    <row r="98" spans="1:3" ht="16" customHeight="1">
+      <c r="A98" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B98" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C98" s="3">
+        <v>2.39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3397,7 +3422,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C97"/>
+  <dimension ref="A1:C98"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4472,6 +4497,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="98" spans="1:3" ht="16" customHeight="1">
+      <c r="A98" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B98" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C98" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4480,7 +4516,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C97"/>
+  <dimension ref="A1:C98"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5555,6 +5591,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="98" spans="1:3" ht="16" customHeight="1">
+      <c r="A98" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B98" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C98" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5563,7 +5610,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C97"/>
+  <dimension ref="A1:C98"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6638,6 +6685,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="98" spans="1:3" ht="16" customHeight="1">
+      <c r="A98" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B98" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C98" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6646,7 +6704,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C97"/>
+  <dimension ref="A1:C98"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7721,6 +7779,17 @@
         <v>6.79</v>
       </c>
     </row>
+    <row r="98" spans="1:3" ht="16" customHeight="1">
+      <c r="A98" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B98" s="3">
+        <v>3.75</v>
+      </c>
+      <c r="C98" s="3">
+        <v>6.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7729,7 +7798,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C97"/>
+  <dimension ref="A1:C98"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8804,6 +8873,17 @@
         <v>4.6933</v>
       </c>
     </row>
+    <row r="98" spans="1:3" ht="16" customHeight="1">
+      <c r="A98" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B98" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C98" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8812,7 +8892,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C97"/>
+  <dimension ref="A1:C98"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9887,6 +9967,17 @@
         <v>3.6842</v>
       </c>
     </row>
+    <row r="98" spans="1:3" ht="16" customHeight="1">
+      <c r="A98" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B98" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C98" s="3">
+        <v>3.6842</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9895,7 +9986,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C97"/>
+  <dimension ref="A1:C98"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10970,6 +11061,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="98" spans="1:3" ht="16" customHeight="1">
+      <c r="A98" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B98" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C98" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10978,7 +11080,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C97"/>
+  <dimension ref="A1:C98"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12053,6 +12155,17 @@
         <v>2.8533</v>
       </c>
     </row>
+    <row r="98" spans="1:3" ht="16" customHeight="1">
+      <c r="A98" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B98" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C98" s="3">
+        <v>3.49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12061,7 +12174,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C97"/>
+  <dimension ref="A1:C98"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13136,6 +13249,17 @@
         <v>2.8667</v>
       </c>
     </row>
+    <row r="98" spans="1:3" ht="16" customHeight="1">
+      <c r="A98" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B98" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C98" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13144,7 +13268,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C97"/>
+  <dimension ref="A1:C98"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14219,6 +14343,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="98" spans="1:3" ht="16" customHeight="1">
+      <c r="A98" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B98" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C98" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-15 15:18:47
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2884" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2904" uniqueCount="102">
   <si>
     <t>Date</t>
   </si>
@@ -328,6 +328,9 @@
   </si>
   <si>
     <t>2026-09-14</t>
+  </si>
+  <si>
+    <t>2026-09-15</t>
   </si>
 </sst>
 </file>
@@ -1234,7 +1237,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C98"/>
+  <dimension ref="A1:C99"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2320,6 +2323,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="99" spans="1:3" ht="16" customHeight="1">
+      <c r="A99" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C99" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2328,7 +2342,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C98"/>
+  <dimension ref="A1:C99"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3414,6 +3428,17 @@
         <v>2.39</v>
       </c>
     </row>
+    <row r="99" spans="1:3" ht="16" customHeight="1">
+      <c r="A99" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B99" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C99" s="3">
+        <v>2.39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3422,7 +3447,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C98"/>
+  <dimension ref="A1:C99"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4508,6 +4533,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="99" spans="1:3" ht="16" customHeight="1">
+      <c r="A99" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B99" s="3">
+        <v>0.92</v>
+      </c>
+      <c r="C99" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4516,7 +4552,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C98"/>
+  <dimension ref="A1:C99"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5602,6 +5638,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="99" spans="1:3" ht="16" customHeight="1">
+      <c r="A99" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C99" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5610,7 +5657,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C98"/>
+  <dimension ref="A1:C99"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6696,6 +6743,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="99" spans="1:3" ht="16" customHeight="1">
+      <c r="A99" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C99" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6704,7 +6762,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C98"/>
+  <dimension ref="A1:C99"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7790,6 +7848,17 @@
         <v>6.79</v>
       </c>
     </row>
+    <row r="99" spans="1:3" ht="16" customHeight="1">
+      <c r="A99" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B99" s="3">
+        <v>3.75</v>
+      </c>
+      <c r="C99" s="3">
+        <v>6.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7798,7 +7867,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C98"/>
+  <dimension ref="A1:C99"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8884,6 +8953,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="99" spans="1:3" ht="16" customHeight="1">
+      <c r="A99" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B99" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C99" s="3">
+        <v>4.0893</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8892,7 +8972,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C98"/>
+  <dimension ref="A1:C99"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9978,6 +10058,17 @@
         <v>3.6842</v>
       </c>
     </row>
+    <row r="99" spans="1:3" ht="16" customHeight="1">
+      <c r="A99" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B99" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C99" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9986,7 +10077,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C98"/>
+  <dimension ref="A1:C99"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11072,6 +11163,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="99" spans="1:3" ht="16" customHeight="1">
+      <c r="A99" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C99" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11080,7 +11182,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C98"/>
+  <dimension ref="A1:C99"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12166,6 +12268,17 @@
         <v>3.49</v>
       </c>
     </row>
+    <row r="99" spans="1:3" ht="16" customHeight="1">
+      <c r="A99" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B99" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C99" s="3">
+        <v>3.1707</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12174,7 +12287,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C98"/>
+  <dimension ref="A1:C99"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13260,6 +13373,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="99" spans="1:3" ht="16" customHeight="1">
+      <c r="A99" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B99" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C99" s="3">
+        <v>2.9867</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13268,7 +13392,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C98"/>
+  <dimension ref="A1:C99"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14354,6 +14478,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="99" spans="1:3" ht="16" customHeight="1">
+      <c r="A99" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C99" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-16 15:11:51
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2904" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2925" uniqueCount="103">
   <si>
     <t>Date</t>
   </si>
@@ -331,6 +331,9 @@
   </si>
   <si>
     <t>2026-09-15</t>
+  </si>
+  <si>
+    <t>2026-09-16</t>
   </si>
 </sst>
 </file>
@@ -1237,7 +1240,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C99"/>
+  <dimension ref="A1:C100"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2334,6 +2337,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="100" spans="1:3" ht="16" customHeight="1">
+      <c r="A100" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B100" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C100" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2342,7 +2356,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C99"/>
+  <dimension ref="A1:C100"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3439,6 +3453,17 @@
         <v>2.39</v>
       </c>
     </row>
+    <row r="100" spans="1:3" ht="16" customHeight="1">
+      <c r="A100" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B100" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C100" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3447,7 +3472,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C99"/>
+  <dimension ref="A1:C100"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4544,6 +4569,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="100" spans="1:3" ht="16" customHeight="1">
+      <c r="A100" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B100" s="3">
+        <v>0.92</v>
+      </c>
+      <c r="C100" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4552,7 +4588,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C99"/>
+  <dimension ref="A1:C100"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5649,6 +5685,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="100" spans="1:3" ht="16" customHeight="1">
+      <c r="A100" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B100" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C100" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5657,7 +5704,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C99"/>
+  <dimension ref="A1:C100"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6754,6 +6801,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="100" spans="1:3" ht="16" customHeight="1">
+      <c r="A100" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B100" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C100" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6762,7 +6820,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C99"/>
+  <dimension ref="A1:C100"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7859,6 +7917,17 @@
         <v>6.79</v>
       </c>
     </row>
+    <row r="100" spans="1:3" ht="16" customHeight="1">
+      <c r="A100" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B100" s="3">
+        <v>3.75</v>
+      </c>
+      <c r="C100" s="3">
+        <v>6.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7867,7 +7936,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C99"/>
+  <dimension ref="A1:C100"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8964,6 +9033,17 @@
         <v>4.0893</v>
       </c>
     </row>
+    <row r="100" spans="1:3" ht="16" customHeight="1">
+      <c r="A100" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B100" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C100" s="3">
+        <v>3.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8972,7 +9052,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C99"/>
+  <dimension ref="A1:C100"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10069,6 +10149,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="100" spans="1:3" ht="16" customHeight="1">
+      <c r="A100" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B100" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C100" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10077,7 +10168,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C99"/>
+  <dimension ref="A1:C100"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11174,6 +11265,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="100" spans="1:3" ht="16" customHeight="1">
+      <c r="A100" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B100" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C100" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11182,7 +11284,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C99"/>
+  <dimension ref="A1:C100"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12279,6 +12381,17 @@
         <v>3.1707</v>
       </c>
     </row>
+    <row r="100" spans="1:3" ht="16" customHeight="1">
+      <c r="A100" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B100" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C100" s="3">
+        <v>3.49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12287,7 +12400,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C99"/>
+  <dimension ref="A1:C100"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13384,6 +13497,17 @@
         <v>2.9867</v>
       </c>
     </row>
+    <row r="100" spans="1:3" ht="16" customHeight="1">
+      <c r="A100" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B100" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C100" s="3">
+        <v>3.0667</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13392,7 +13516,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C99"/>
+  <dimension ref="A1:C100"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14489,6 +14613,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="100" spans="1:3" ht="16" customHeight="1">
+      <c r="A100" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B100" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C100" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-17 15:20:47
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2925" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2944" uniqueCount="104">
   <si>
     <t>Date</t>
   </si>
@@ -334,6 +334,9 @@
   </si>
   <si>
     <t>2026-09-16</t>
+  </si>
+  <si>
+    <t>2026-09-17</t>
   </si>
 </sst>
 </file>
@@ -1240,7 +1243,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C100"/>
+  <dimension ref="A1:C101"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2348,6 +2351,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="101" spans="1:3" ht="16" customHeight="1">
+      <c r="A101" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B101" s="3">
+        <v>7.805</v>
+      </c>
+      <c r="C101" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2356,7 +2370,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C100"/>
+  <dimension ref="A1:C101"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3464,6 +3478,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="101" spans="1:3" ht="16" customHeight="1">
+      <c r="A101" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B101" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C101" s="3">
+        <v>2.39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3472,7 +3497,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C100"/>
+  <dimension ref="A1:C101"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4580,6 +4605,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="101" spans="1:3" ht="16" customHeight="1">
+      <c r="A101" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B101" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C101" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4588,7 +4624,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C100"/>
+  <dimension ref="A1:C101"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5696,6 +5732,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="101" spans="1:3" ht="16" customHeight="1">
+      <c r="A101" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C101" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5704,7 +5751,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C100"/>
+  <dimension ref="A1:C101"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6812,6 +6859,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="101" spans="1:3" ht="16" customHeight="1">
+      <c r="A101" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C101" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6820,7 +6878,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C100"/>
+  <dimension ref="A1:C101"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7928,6 +7986,17 @@
         <v>6.79</v>
       </c>
     </row>
+    <row r="101" spans="1:3" ht="16" customHeight="1">
+      <c r="A101" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B101" s="3">
+        <v>3.75</v>
+      </c>
+      <c r="C101" s="3">
+        <v>6.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7936,7 +8005,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C100"/>
+  <dimension ref="A1:C101"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9044,6 +9113,17 @@
         <v>3.79</v>
       </c>
     </row>
+    <row r="101" spans="1:3" ht="16" customHeight="1">
+      <c r="A101" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B101" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C101" s="3">
+        <v>5.4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9052,7 +9132,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C100"/>
+  <dimension ref="A1:C101"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10160,6 +10240,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="101" spans="1:3" ht="16" customHeight="1">
+      <c r="A101" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B101" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C101" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10168,7 +10259,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C100"/>
+  <dimension ref="A1:C101"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11276,6 +11367,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="101" spans="1:3" ht="16" customHeight="1">
+      <c r="A101" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B101" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C101" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11284,7 +11386,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C100"/>
+  <dimension ref="A1:C101"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12392,6 +12494,17 @@
         <v>3.49</v>
       </c>
     </row>
+    <row r="101" spans="1:3" ht="16" customHeight="1">
+      <c r="A101" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B101" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C101" s="3">
+        <v>3.49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12400,7 +12513,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C100"/>
+  <dimension ref="A1:C101"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13508,6 +13621,17 @@
         <v>3.0667</v>
       </c>
     </row>
+    <row r="101" spans="1:3" ht="16" customHeight="1">
+      <c r="A101" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B101" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C101" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13516,7 +13640,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C100"/>
+  <dimension ref="A1:C101"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14624,6 +14748,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="101" spans="1:3" ht="16" customHeight="1">
+      <c r="A101" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C101" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-18 14:41:04
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2944" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2965" uniqueCount="105">
   <si>
     <t>Date</t>
   </si>
@@ -337,6 +337,9 @@
   </si>
   <si>
     <t>2026-09-17</t>
+  </si>
+  <si>
+    <t>2026-09-18</t>
   </si>
 </sst>
 </file>
@@ -1243,7 +1246,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C101"/>
+  <dimension ref="A1:C102"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2362,6 +2365,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="102" spans="1:3" ht="16" customHeight="1">
+      <c r="A102" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C102" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2370,7 +2384,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C101"/>
+  <dimension ref="A1:C102"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3489,6 +3503,17 @@
         <v>2.39</v>
       </c>
     </row>
+    <row r="102" spans="1:3" ht="16" customHeight="1">
+      <c r="A102" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B102" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C102" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3497,7 +3522,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C101"/>
+  <dimension ref="A1:C102"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4616,6 +4641,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="102" spans="1:3" ht="16" customHeight="1">
+      <c r="A102" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B102" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C102" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4624,7 +4660,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C101"/>
+  <dimension ref="A1:C102"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5743,6 +5779,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="102" spans="1:3" ht="16" customHeight="1">
+      <c r="A102" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C102" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5751,7 +5798,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C101"/>
+  <dimension ref="A1:C102"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6870,6 +6917,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="102" spans="1:3" ht="16" customHeight="1">
+      <c r="A102" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C102" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6878,7 +6936,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C101"/>
+  <dimension ref="A1:C102"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7997,6 +8055,17 @@
         <v>6.79</v>
       </c>
     </row>
+    <row r="102" spans="1:3" ht="16" customHeight="1">
+      <c r="A102" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B102" s="3">
+        <v>3.75</v>
+      </c>
+      <c r="C102" s="3">
+        <v>6.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8005,7 +8074,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C101"/>
+  <dimension ref="A1:C102"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9124,6 +9193,17 @@
         <v>5.4</v>
       </c>
     </row>
+    <row r="102" spans="1:3" ht="16" customHeight="1">
+      <c r="A102" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B102" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C102" s="3">
+        <v>3.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9132,7 +9212,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C101"/>
+  <dimension ref="A1:C102"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10251,6 +10331,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="102" spans="1:3" ht="16" customHeight="1">
+      <c r="A102" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B102" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C102" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10259,7 +10350,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C101"/>
+  <dimension ref="A1:C102"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11378,6 +11469,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="102" spans="1:3" ht="16" customHeight="1">
+      <c r="A102" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C102" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11386,7 +11488,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C101"/>
+  <dimension ref="A1:C102"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12505,6 +12607,17 @@
         <v>3.49</v>
       </c>
     </row>
+    <row r="102" spans="1:3" ht="16" customHeight="1">
+      <c r="A102" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B102" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C102" s="3">
+        <v>3.49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12513,7 +12626,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C101"/>
+  <dimension ref="A1:C102"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13632,6 +13745,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="102" spans="1:3" ht="16" customHeight="1">
+      <c r="A102" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B102" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C102" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13640,7 +13764,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C101"/>
+  <dimension ref="A1:C102"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14759,6 +14883,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="102" spans="1:3" ht="16" customHeight="1">
+      <c r="A102" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C102" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-19 14:01:22
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2965" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2985" uniqueCount="106">
   <si>
     <t>Date</t>
   </si>
@@ -340,6 +340,9 @@
   </si>
   <si>
     <t>2026-09-18</t>
+  </si>
+  <si>
+    <t>2026-09-19</t>
   </si>
 </sst>
 </file>
@@ -1246,7 +1249,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C102"/>
+  <dimension ref="A1:C103"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2376,6 +2379,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="103" spans="1:3" ht="16" customHeight="1">
+      <c r="A103" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C103" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2384,7 +2398,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C102"/>
+  <dimension ref="A1:C103"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3514,6 +3528,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="103" spans="1:3" ht="16" customHeight="1">
+      <c r="A103" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B103" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C103" s="3">
+        <v>2.39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3522,7 +3547,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C102"/>
+  <dimension ref="A1:C103"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4652,6 +4677,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="103" spans="1:3" ht="16" customHeight="1">
+      <c r="A103" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B103" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C103" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4660,7 +4696,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C102"/>
+  <dimension ref="A1:C103"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5790,6 +5826,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="103" spans="1:3" ht="16" customHeight="1">
+      <c r="A103" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C103" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5798,7 +5845,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C102"/>
+  <dimension ref="A1:C103"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6928,6 +6975,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="103" spans="1:3" ht="16" customHeight="1">
+      <c r="A103" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C103" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6936,7 +6994,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C102"/>
+  <dimension ref="A1:C103"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8066,6 +8124,17 @@
         <v>6.79</v>
       </c>
     </row>
+    <row r="103" spans="1:3" ht="16" customHeight="1">
+      <c r="A103" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B103" s="3">
+        <v>3.75</v>
+      </c>
+      <c r="C103" s="3">
+        <v>6.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8074,7 +8143,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C102"/>
+  <dimension ref="A1:C103"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9204,6 +9273,17 @@
         <v>3.79</v>
       </c>
     </row>
+    <row r="103" spans="1:3" ht="16" customHeight="1">
+      <c r="A103" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B103" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C103" s="3">
+        <v>5.032</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9212,7 +9292,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C102"/>
+  <dimension ref="A1:C103"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10342,6 +10422,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="103" spans="1:3" ht="16" customHeight="1">
+      <c r="A103" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B103" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C103" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10350,7 +10441,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C102"/>
+  <dimension ref="A1:C103"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11480,6 +11571,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="103" spans="1:3" ht="16" customHeight="1">
+      <c r="A103" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C103" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11488,7 +11590,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C102"/>
+  <dimension ref="A1:C103"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12618,6 +12720,17 @@
         <v>3.49</v>
       </c>
     </row>
+    <row r="103" spans="1:3" ht="16" customHeight="1">
+      <c r="A103" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B103" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C103" s="3">
+        <v>3.49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12626,7 +12739,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C102"/>
+  <dimension ref="A1:C103"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13756,6 +13869,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="103" spans="1:3" ht="16" customHeight="1">
+      <c r="A103" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B103" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C103" s="3">
+        <v>3.1466</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13764,7 +13888,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C102"/>
+  <dimension ref="A1:C103"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14894,6 +15018,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="103" spans="1:3" ht="16" customHeight="1">
+      <c r="A103" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C103" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-20 14:22:23
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2985" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3005" uniqueCount="107">
   <si>
     <t>Date</t>
   </si>
@@ -343,6 +343,9 @@
   </si>
   <si>
     <t>2026-09-19</t>
+  </si>
+  <si>
+    <t>2026-09-20</t>
   </si>
 </sst>
 </file>
@@ -1249,7 +1252,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C103"/>
+  <dimension ref="A1:C104"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2390,6 +2393,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="104" spans="1:3" ht="16" customHeight="1">
+      <c r="A104" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B104" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C104" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2398,7 +2412,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C103"/>
+  <dimension ref="A1:C104"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3539,6 +3553,17 @@
         <v>2.39</v>
       </c>
     </row>
+    <row r="104" spans="1:3" ht="16" customHeight="1">
+      <c r="A104" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B104" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C104" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3547,7 +3572,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C103"/>
+  <dimension ref="A1:C104"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4688,6 +4713,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="104" spans="1:3" ht="16" customHeight="1">
+      <c r="A104" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B104" s="3">
+        <v>0.92</v>
+      </c>
+      <c r="C104" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4696,7 +4732,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C103"/>
+  <dimension ref="A1:C104"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5837,6 +5873,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="104" spans="1:3" ht="16" customHeight="1">
+      <c r="A104" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B104" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C104" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5845,7 +5892,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C103"/>
+  <dimension ref="A1:C104"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6986,6 +7033,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="104" spans="1:3" ht="16" customHeight="1">
+      <c r="A104" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B104" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C104" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6994,7 +7052,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C103"/>
+  <dimension ref="A1:C104"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8135,6 +8193,17 @@
         <v>6.79</v>
       </c>
     </row>
+    <row r="104" spans="1:3" ht="16" customHeight="1">
+      <c r="A104" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B104" s="3">
+        <v>3.75</v>
+      </c>
+      <c r="C104" s="3">
+        <v>6.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8143,7 +8212,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C103"/>
+  <dimension ref="A1:C104"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9284,6 +9353,17 @@
         <v>5.032</v>
       </c>
     </row>
+    <row r="104" spans="1:3" ht="16" customHeight="1">
+      <c r="A104" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B104" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C104" s="3">
+        <v>4.1693</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9292,7 +9372,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C103"/>
+  <dimension ref="A1:C104"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10433,6 +10513,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="104" spans="1:3" ht="16" customHeight="1">
+      <c r="A104" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B104" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C104" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10441,7 +10532,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C103"/>
+  <dimension ref="A1:C104"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11582,6 +11673,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="104" spans="1:3" ht="16" customHeight="1">
+      <c r="A104" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B104" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C104" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11590,7 +11692,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C103"/>
+  <dimension ref="A1:C104"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12731,6 +12833,17 @@
         <v>3.49</v>
       </c>
     </row>
+    <row r="104" spans="1:3" ht="16" customHeight="1">
+      <c r="A104" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B104" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C104" s="3">
+        <v>3.49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12739,7 +12852,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C103"/>
+  <dimension ref="A1:C104"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13880,6 +13993,17 @@
         <v>3.1466</v>
       </c>
     </row>
+    <row r="104" spans="1:3" ht="16" customHeight="1">
+      <c r="A104" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B104" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C104" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13888,7 +14012,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C103"/>
+  <dimension ref="A1:C104"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15029,6 +15153,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="104" spans="1:3" ht="16" customHeight="1">
+      <c r="A104" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B104" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C104" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-21 16:41:25
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3005" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3024" uniqueCount="108">
   <si>
     <t>Date</t>
   </si>
@@ -346,6 +346,9 @@
   </si>
   <si>
     <t>2026-09-20</t>
+  </si>
+  <si>
+    <t>2026-09-21</t>
   </si>
 </sst>
 </file>
@@ -1252,7 +1255,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C104"/>
+  <dimension ref="A1:C105"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2404,6 +2407,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="105" spans="1:3" ht="16" customHeight="1">
+      <c r="A105" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C105" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2412,7 +2426,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C104"/>
+  <dimension ref="A1:C105"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3564,6 +3578,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="105" spans="1:3" ht="16" customHeight="1">
+      <c r="A105" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B105" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C105" s="3">
+        <v>2.39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3572,7 +3597,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C104"/>
+  <dimension ref="A1:C105"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4724,6 +4749,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="105" spans="1:3" ht="16" customHeight="1">
+      <c r="A105" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B105" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C105" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4732,7 +4768,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C104"/>
+  <dimension ref="A1:C105"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5884,6 +5920,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="105" spans="1:3" ht="16" customHeight="1">
+      <c r="A105" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C105" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5892,7 +5939,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C104"/>
+  <dimension ref="A1:C105"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7044,6 +7091,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="105" spans="1:3" ht="16" customHeight="1">
+      <c r="A105" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C105" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7052,7 +7110,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C104"/>
+  <dimension ref="A1:C105"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8204,6 +8262,17 @@
         <v>6.79</v>
       </c>
     </row>
+    <row r="105" spans="1:3" ht="16" customHeight="1">
+      <c r="A105" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B105" s="3">
+        <v>3.75</v>
+      </c>
+      <c r="C105" s="3">
+        <v>6.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8212,7 +8281,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C104"/>
+  <dimension ref="A1:C105"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9364,6 +9433,17 @@
         <v>4.1693</v>
       </c>
     </row>
+    <row r="105" spans="1:3" ht="16" customHeight="1">
+      <c r="A105" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B105" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C105" s="3">
+        <v>5.4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9372,7 +9452,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C104"/>
+  <dimension ref="A1:C105"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10524,6 +10604,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="105" spans="1:3" ht="16" customHeight="1">
+      <c r="A105" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B105" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C105" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10532,7 +10623,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C104"/>
+  <dimension ref="A1:C105"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11684,6 +11775,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="105" spans="1:3" ht="16" customHeight="1">
+      <c r="A105" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B105" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C105" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11692,7 +11794,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C104"/>
+  <dimension ref="A1:C105"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12844,6 +12946,17 @@
         <v>3.49</v>
       </c>
     </row>
+    <row r="105" spans="1:3" ht="16" customHeight="1">
+      <c r="A105" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B105" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C105" s="3">
+        <v>3.49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12852,7 +12965,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C104"/>
+  <dimension ref="A1:C105"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14004,6 +14117,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="105" spans="1:3" ht="16" customHeight="1">
+      <c r="A105" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B105" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C105" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14012,7 +14136,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C104"/>
+  <dimension ref="A1:C105"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15164,6 +15288,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="105" spans="1:3" ht="16" customHeight="1">
+      <c r="A105" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C105" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-22 15:12:50
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3024" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3044" uniqueCount="109">
   <si>
     <t>Date</t>
   </si>
@@ -350,6 +350,9 @@
   <si>
     <t>2026-09-21</t>
   </si>
+  <si>
+    <t>2026-09-22</t>
+  </si>
 </sst>
 </file>
 
@@ -465,7 +468,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -485,7 +488,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -508,7 +511,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -528,7 +531,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -551,7 +554,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -571,7 +574,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -594,7 +597,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -614,7 +617,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -680,7 +683,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -700,7 +703,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -723,7 +726,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -743,7 +746,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -766,7 +769,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -786,7 +789,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -809,7 +812,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -829,7 +832,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -852,7 +855,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -872,7 +875,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -895,7 +898,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -915,7 +918,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1255,7 +1258,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C105"/>
+  <dimension ref="A1:C106"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2418,6 +2421,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="106" spans="1:3" ht="16" customHeight="1">
+      <c r="A106" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B106" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C106" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2426,7 +2440,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C105"/>
+  <dimension ref="A1:C106"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3589,6 +3603,17 @@
         <v>2.39</v>
       </c>
     </row>
+    <row r="106" spans="1:3" ht="16" customHeight="1">
+      <c r="A106" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B106" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C106" s="3">
+        <v>2.39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3597,7 +3622,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C105"/>
+  <dimension ref="A1:C106"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4760,6 +4785,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="106" spans="1:3" ht="16" customHeight="1">
+      <c r="A106" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B106" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C106" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4768,7 +4804,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C105"/>
+  <dimension ref="A1:C106"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5931,6 +5967,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="106" spans="1:3" ht="16" customHeight="1">
+      <c r="A106" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B106" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C106" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5939,7 +5986,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C105"/>
+  <dimension ref="A1:C106"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7102,6 +7149,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="106" spans="1:3" ht="16" customHeight="1">
+      <c r="A106" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B106" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C106" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7110,7 +7168,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C105"/>
+  <dimension ref="A1:C106"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8273,6 +8331,17 @@
         <v>6.79</v>
       </c>
     </row>
+    <row r="106" spans="1:3" ht="16" customHeight="1">
+      <c r="A106" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B106" s="3">
+        <v>3.75</v>
+      </c>
+      <c r="C106" s="3">
+        <v>6.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8281,7 +8350,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C105"/>
+  <dimension ref="A1:C106"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9444,6 +9513,17 @@
         <v>5.4</v>
       </c>
     </row>
+    <row r="106" spans="1:3" ht="16" customHeight="1">
+      <c r="A106" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B106" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C106" s="3">
+        <v>5.6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9452,7 +9532,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C105"/>
+  <dimension ref="A1:C106"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10615,6 +10695,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="106" spans="1:3" ht="16" customHeight="1">
+      <c r="A106" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B106" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C106" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10623,7 +10714,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C105"/>
+  <dimension ref="A1:C106"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11786,6 +11877,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="106" spans="1:3" ht="16" customHeight="1">
+      <c r="A106" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B106" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C106" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11794,7 +11896,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C105"/>
+  <dimension ref="A1:C106"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12957,6 +13059,17 @@
         <v>3.49</v>
       </c>
     </row>
+    <row r="106" spans="1:3" ht="16" customHeight="1">
+      <c r="A106" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B106" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C106" s="3">
+        <v>3.49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12965,7 +13078,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C105"/>
+  <dimension ref="A1:C106"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14128,6 +14241,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="106" spans="1:3" ht="16" customHeight="1">
+      <c r="A106" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B106" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C106" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14136,7 +14260,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C105"/>
+  <dimension ref="A1:C106"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15299,6 +15423,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="106" spans="1:3" ht="16" customHeight="1">
+      <c r="A106" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B106" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C106" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-23 15:12:56
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3044" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3066" uniqueCount="110">
   <si>
     <t>Date</t>
   </si>
@@ -353,6 +353,9 @@
   <si>
     <t>2026-09-22</t>
   </si>
+  <si>
+    <t>2026-09-23</t>
+  </si>
 </sst>
 </file>
 
@@ -468,7 +471,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>65821</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -488,7 +491,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="7990621" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -511,7 +514,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>65821</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -531,7 +534,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="7990621" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -554,7 +557,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>65821</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -574,7 +577,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="7990621" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -597,7 +600,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>65821</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -617,7 +620,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="7990621" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -683,7 +686,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>65821</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -703,7 +706,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="7990621" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -726,7 +729,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>65821</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -746,7 +749,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="7990621" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -769,7 +772,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>65821</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -789,7 +792,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="7990621" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -812,7 +815,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>65821</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -832,7 +835,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="7990621" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -855,7 +858,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>65821</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -875,7 +878,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="7990621" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -898,7 +901,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>65821</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -918,7 +921,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="7990621" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1258,7 +1261,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C106"/>
+  <dimension ref="A1:C107"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2432,6 +2435,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="107" spans="1:3" ht="16" customHeight="1">
+      <c r="A107" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C107" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2440,7 +2454,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C106"/>
+  <dimension ref="A1:C107"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3614,6 +3628,17 @@
         <v>2.39</v>
       </c>
     </row>
+    <row r="107" spans="1:3" ht="16" customHeight="1">
+      <c r="A107" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B107" s="3">
+        <v>3.39</v>
+      </c>
+      <c r="C107" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3622,7 +3647,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C106"/>
+  <dimension ref="A1:C107"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4796,6 +4821,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="107" spans="1:3" ht="16" customHeight="1">
+      <c r="A107" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B107" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C107" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4804,7 +4840,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C106"/>
+  <dimension ref="A1:C107"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5978,6 +6014,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="107" spans="1:3" ht="16" customHeight="1">
+      <c r="A107" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C107" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5986,7 +6033,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C106"/>
+  <dimension ref="A1:C107"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7160,6 +7207,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="107" spans="1:3" ht="16" customHeight="1">
+      <c r="A107" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C107" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7168,7 +7226,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C106"/>
+  <dimension ref="A1:C107"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8342,6 +8400,17 @@
         <v>6.79</v>
       </c>
     </row>
+    <row r="107" spans="1:3" ht="16" customHeight="1">
+      <c r="A107" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B107" s="3">
+        <v>3.75</v>
+      </c>
+      <c r="C107" s="3">
+        <v>6.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8350,7 +8419,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C106"/>
+  <dimension ref="A1:C107"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9524,6 +9593,17 @@
         <v>5.6</v>
       </c>
     </row>
+    <row r="107" spans="1:3" ht="16" customHeight="1">
+      <c r="A107" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B107" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C107" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9532,7 +9612,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C106"/>
+  <dimension ref="A1:C107"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10706,6 +10786,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="107" spans="1:3" ht="16" customHeight="1">
+      <c r="A107" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B107" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C107" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10714,7 +10805,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C106"/>
+  <dimension ref="A1:C107"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11888,6 +11979,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="107" spans="1:3" ht="16" customHeight="1">
+      <c r="A107" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C107" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11896,7 +11998,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C106"/>
+  <dimension ref="A1:C107"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13070,6 +13172,17 @@
         <v>3.49</v>
       </c>
     </row>
+    <row r="107" spans="1:3" ht="16" customHeight="1">
+      <c r="A107" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B107" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C107" s="3">
+        <v>3.49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13078,7 +13191,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C106"/>
+  <dimension ref="A1:C107"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14252,6 +14365,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="107" spans="1:3" ht="16" customHeight="1">
+      <c r="A107" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B107" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C107" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14260,7 +14384,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C106"/>
+  <dimension ref="A1:C107"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15434,6 +15558,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="107" spans="1:3" ht="16" customHeight="1">
+      <c r="A107" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C107" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-24 15:32:29
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3066" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3087" uniqueCount="111">
   <si>
     <t>Date</t>
   </si>
@@ -356,6 +356,9 @@
   <si>
     <t>2026-09-23</t>
   </si>
+  <si>
+    <t>2026-09-24</t>
+  </si>
 </sst>
 </file>
 
@@ -471,7 +474,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>65821</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -491,7 +494,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7990621" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -514,7 +517,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>65821</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -534,7 +537,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7990621" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -557,7 +560,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>65821</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -577,7 +580,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7990621" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -600,7 +603,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>65821</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -620,7 +623,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7990621" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -686,7 +689,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>65821</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -706,7 +709,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7990621" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -729,7 +732,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>65821</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -749,7 +752,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7990621" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -772,7 +775,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>65821</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -792,7 +795,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7990621" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -815,7 +818,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>65821</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -835,7 +838,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7990621" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -858,7 +861,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>65821</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -878,7 +881,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7990621" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -901,7 +904,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>65821</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -921,7 +924,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7990621" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1261,7 +1264,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C107"/>
+  <dimension ref="A1:C108"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2446,6 +2449,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="108" spans="1:3" ht="16" customHeight="1">
+      <c r="A108" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B108" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C108" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2454,7 +2468,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C107"/>
+  <dimension ref="A1:C108"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3639,6 +3653,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="108" spans="1:3" ht="16" customHeight="1">
+      <c r="A108" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B108" s="3">
+        <v>3.39</v>
+      </c>
+      <c r="C108" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3647,7 +3672,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C107"/>
+  <dimension ref="A1:C108"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4832,6 +4857,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="108" spans="1:3" ht="16" customHeight="1">
+      <c r="A108" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B108" s="3">
+        <v>0.92</v>
+      </c>
+      <c r="C108" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4840,7 +4876,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C107"/>
+  <dimension ref="A1:C108"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6025,6 +6061,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="108" spans="1:3" ht="16" customHeight="1">
+      <c r="A108" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B108" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C108" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6033,7 +6080,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C107"/>
+  <dimension ref="A1:C108"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7218,6 +7265,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="108" spans="1:3" ht="16" customHeight="1">
+      <c r="A108" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B108" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C108" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7226,7 +7284,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C107"/>
+  <dimension ref="A1:C108"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8411,6 +8469,17 @@
         <v>6.79</v>
       </c>
     </row>
+    <row r="108" spans="1:3" ht="16" customHeight="1">
+      <c r="A108" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B108" s="3">
+        <v>3.75</v>
+      </c>
+      <c r="C108" s="3">
+        <v>9.375</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8419,7 +8488,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C107"/>
+  <dimension ref="A1:C108"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9604,6 +9673,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="108" spans="1:3" ht="16" customHeight="1">
+      <c r="A108" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B108" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C108" s="3">
+        <v>5.4667</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9612,7 +9692,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C107"/>
+  <dimension ref="A1:C108"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10797,6 +10877,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="108" spans="1:3" ht="16" customHeight="1">
+      <c r="A108" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B108" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C108" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10805,7 +10896,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C107"/>
+  <dimension ref="A1:C108"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11990,6 +12081,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="108" spans="1:3" ht="16" customHeight="1">
+      <c r="A108" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B108" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C108" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11998,7 +12100,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C107"/>
+  <dimension ref="A1:C108"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13183,6 +13285,17 @@
         <v>3.49</v>
       </c>
     </row>
+    <row r="108" spans="1:3" ht="16" customHeight="1">
+      <c r="A108" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B108" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C108" s="3">
+        <v>3.49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13191,7 +13304,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C107"/>
+  <dimension ref="A1:C108"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14376,6 +14489,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="108" spans="1:3" ht="16" customHeight="1">
+      <c r="A108" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B108" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C108" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14384,7 +14508,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C107"/>
+  <dimension ref="A1:C108"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15569,6 +15693,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="108" spans="1:3" ht="16" customHeight="1">
+      <c r="A108" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B108" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C108" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-25 15:36:38
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3087" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3109" uniqueCount="112">
   <si>
     <t>Date</t>
   </si>
@@ -358,6 +358,9 @@
   </si>
   <si>
     <t>2026-09-24</t>
+  </si>
+  <si>
+    <t>2026-09-25</t>
   </si>
 </sst>
 </file>
@@ -1264,7 +1267,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C108"/>
+  <dimension ref="A1:C109"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2460,6 +2463,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="109" spans="1:3" ht="16" customHeight="1">
+      <c r="A109" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C109" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2468,7 +2482,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C108"/>
+  <dimension ref="A1:C109"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3664,6 +3678,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="109" spans="1:3" ht="16" customHeight="1">
+      <c r="A109" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C109" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3672,7 +3697,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C108"/>
+  <dimension ref="A1:C109"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4868,6 +4893,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="109" spans="1:3" ht="16" customHeight="1">
+      <c r="A109" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B109" s="3">
+        <v>0.92</v>
+      </c>
+      <c r="C109" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4876,7 +4912,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C108"/>
+  <dimension ref="A1:C109"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6072,6 +6108,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="109" spans="1:3" ht="16" customHeight="1">
+      <c r="A109" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C109" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6080,7 +6127,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C108"/>
+  <dimension ref="A1:C109"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7276,6 +7323,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="109" spans="1:3" ht="16" customHeight="1">
+      <c r="A109" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C109" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7284,7 +7342,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C108"/>
+  <dimension ref="A1:C109"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8480,6 +8538,17 @@
         <v>9.375</v>
       </c>
     </row>
+    <row r="109" spans="1:3" ht="16" customHeight="1">
+      <c r="A109" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B109" s="3">
+        <v>3.75</v>
+      </c>
+      <c r="C109" s="3">
+        <v>6.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8488,7 +8557,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C108"/>
+  <dimension ref="A1:C109"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9684,6 +9753,17 @@
         <v>5.4667</v>
       </c>
     </row>
+    <row r="109" spans="1:3" ht="16" customHeight="1">
+      <c r="A109" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B109" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C109" s="3">
+        <v>5.4333</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9692,7 +9772,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C108"/>
+  <dimension ref="A1:C109"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10888,6 +10968,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="109" spans="1:3" ht="16" customHeight="1">
+      <c r="A109" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B109" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C109" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10896,7 +10987,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C108"/>
+  <dimension ref="A1:C109"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12092,6 +12183,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="109" spans="1:3" ht="16" customHeight="1">
+      <c r="A109" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C109" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12100,7 +12202,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C108"/>
+  <dimension ref="A1:C109"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13296,6 +13398,17 @@
         <v>3.49</v>
       </c>
     </row>
+    <row r="109" spans="1:3" ht="16" customHeight="1">
+      <c r="A109" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B109" s="3">
+        <v>2.89</v>
+      </c>
+      <c r="C109" s="3">
+        <v>3.1053</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13304,7 +13417,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C108"/>
+  <dimension ref="A1:C109"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14500,6 +14613,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="109" spans="1:3" ht="16" customHeight="1">
+      <c r="A109" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B109" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C109" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14508,7 +14632,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C108"/>
+  <dimension ref="A1:C109"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15704,6 +15828,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="109" spans="1:3" ht="16" customHeight="1">
+      <c r="A109" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C109" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-26 14:47:07
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3109" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3128" uniqueCount="113">
   <si>
     <t>Date</t>
   </si>
@@ -361,6 +361,9 @@
   </si>
   <si>
     <t>2026-09-25</t>
+  </si>
+  <si>
+    <t>2026-09-26</t>
   </si>
 </sst>
 </file>
@@ -1267,7 +1270,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C109"/>
+  <dimension ref="A1:C110"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2474,6 +2477,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="110" spans="1:3" ht="16" customHeight="1">
+      <c r="A110" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B110" s="3">
+        <v>7.99</v>
+      </c>
+      <c r="C110" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2482,7 +2496,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C109"/>
+  <dimension ref="A1:C110"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3689,6 +3703,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="110" spans="1:3" ht="16" customHeight="1">
+      <c r="A110" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B110" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C110" s="3">
+        <v>2.39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3697,7 +3722,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C109"/>
+  <dimension ref="A1:C110"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4904,6 +4929,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="110" spans="1:3" ht="16" customHeight="1">
+      <c r="A110" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B110" s="3">
+        <v>0.92</v>
+      </c>
+      <c r="C110" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4912,7 +4948,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C109"/>
+  <dimension ref="A1:C110"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6119,6 +6155,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="110" spans="1:3" ht="16" customHeight="1">
+      <c r="A110" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B110" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C110" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6127,7 +6174,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C109"/>
+  <dimension ref="A1:C110"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7334,6 +7381,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="110" spans="1:3" ht="16" customHeight="1">
+      <c r="A110" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B110" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C110" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7342,7 +7400,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C109"/>
+  <dimension ref="A1:C110"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8549,6 +8607,17 @@
         <v>6.79</v>
       </c>
     </row>
+    <row r="110" spans="1:3" ht="16" customHeight="1">
+      <c r="A110" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B110" s="3">
+        <v>6.95</v>
+      </c>
+      <c r="C110" s="3">
+        <v>6.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8557,7 +8626,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C109"/>
+  <dimension ref="A1:C110"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9764,6 +9833,17 @@
         <v>5.4333</v>
       </c>
     </row>
+    <row r="110" spans="1:3" ht="16" customHeight="1">
+      <c r="A110" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B110" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C110" s="3">
+        <v>3.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9772,7 +9852,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C109"/>
+  <dimension ref="A1:C110"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10979,6 +11059,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="110" spans="1:3" ht="16" customHeight="1">
+      <c r="A110" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B110" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C110" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10987,7 +11078,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C109"/>
+  <dimension ref="A1:C110"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12194,6 +12285,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="110" spans="1:3" ht="16" customHeight="1">
+      <c r="A110" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B110" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C110" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12202,7 +12304,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C109"/>
+  <dimension ref="A1:C110"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13409,6 +13511,17 @@
         <v>3.1053</v>
       </c>
     </row>
+    <row r="110" spans="1:3" ht="16" customHeight="1">
+      <c r="A110" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B110" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C110" s="3">
+        <v>2.7453</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13417,7 +13530,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C109"/>
+  <dimension ref="A1:C110"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14624,6 +14737,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="110" spans="1:3" ht="16" customHeight="1">
+      <c r="A110" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B110" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C110" s="3">
+        <v>2.8106</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14632,7 +14756,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C109"/>
+  <dimension ref="A1:C110"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15839,6 +15963,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="110" spans="1:3" ht="16" customHeight="1">
+      <c r="A110" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B110" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C110" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-27 15:25:06
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3128" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3150" uniqueCount="114">
   <si>
     <t>Date</t>
   </si>
@@ -364,6 +364,9 @@
   </si>
   <si>
     <t>2026-09-26</t>
+  </si>
+  <si>
+    <t>2026-09-27</t>
   </si>
 </sst>
 </file>
@@ -1270,7 +1273,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C110"/>
+  <dimension ref="A1:C111"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2488,6 +2491,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="111" spans="1:3" ht="16" customHeight="1">
+      <c r="A111" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B111" s="3">
+        <v>7.99</v>
+      </c>
+      <c r="C111" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2496,7 +2510,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C110"/>
+  <dimension ref="A1:C111"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3714,6 +3728,17 @@
         <v>2.39</v>
       </c>
     </row>
+    <row r="111" spans="1:3" ht="16" customHeight="1">
+      <c r="A111" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C111" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3722,7 +3747,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C110"/>
+  <dimension ref="A1:C111"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4940,6 +4965,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="111" spans="1:3" ht="16" customHeight="1">
+      <c r="A111" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B111" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C111" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4948,7 +4984,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C110"/>
+  <dimension ref="A1:C111"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6166,6 +6202,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="111" spans="1:3" ht="16" customHeight="1">
+      <c r="A111" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C111" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6174,7 +6221,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C110"/>
+  <dimension ref="A1:C111"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7392,6 +7439,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="111" spans="1:3" ht="16" customHeight="1">
+      <c r="A111" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C111" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7400,7 +7458,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C110"/>
+  <dimension ref="A1:C111"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8618,6 +8676,17 @@
         <v>6.79</v>
       </c>
     </row>
+    <row r="111" spans="1:3" ht="16" customHeight="1">
+      <c r="A111" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B111" s="3">
+        <v>6.49</v>
+      </c>
+      <c r="C111" s="3">
+        <v>6.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8626,7 +8695,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C110"/>
+  <dimension ref="A1:C111"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9844,6 +9913,17 @@
         <v>3.79</v>
       </c>
     </row>
+    <row r="111" spans="1:3" ht="16" customHeight="1">
+      <c r="A111" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B111" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C111" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9852,7 +9932,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C110"/>
+  <dimension ref="A1:C111"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11070,6 +11150,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="111" spans="1:3" ht="16" customHeight="1">
+      <c r="A111" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B111" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C111" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11078,7 +11169,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C110"/>
+  <dimension ref="A1:C111"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12296,6 +12387,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="111" spans="1:3" ht="16" customHeight="1">
+      <c r="A111" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C111" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12304,7 +12406,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C110"/>
+  <dimension ref="A1:C111"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13522,6 +13624,17 @@
         <v>2.7453</v>
       </c>
     </row>
+    <row r="111" spans="1:3" ht="16" customHeight="1">
+      <c r="A111" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B111" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C111" s="3">
+        <v>3.3453</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13530,7 +13643,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C110"/>
+  <dimension ref="A1:C111"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14748,6 +14861,17 @@
         <v>2.8106</v>
       </c>
     </row>
+    <row r="111" spans="1:3" ht="16" customHeight="1">
+      <c r="A111" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B111" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C111" s="3">
+        <v>3.1066</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14756,7 +14880,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C110"/>
+  <dimension ref="A1:C111"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15974,6 +16098,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="111" spans="1:3" ht="16" customHeight="1">
+      <c r="A111" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C111" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-28 18:17:46
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3150" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3171" uniqueCount="115">
   <si>
     <t>Date</t>
   </si>
@@ -367,6 +367,9 @@
   </si>
   <si>
     <t>2026-09-27</t>
+  </si>
+  <si>
+    <t>2026-09-28</t>
   </si>
 </sst>
 </file>
@@ -1273,7 +1276,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C111"/>
+  <dimension ref="A1:C112"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2502,6 +2505,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="112" spans="1:3" ht="16" customHeight="1">
+      <c r="A112" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B112" s="3">
+        <v>8.6212</v>
+      </c>
+      <c r="C112" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2510,7 +2524,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C111"/>
+  <dimension ref="A1:C112"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3739,6 +3753,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="112" spans="1:3" ht="16" customHeight="1">
+      <c r="A112" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B112" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C112" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3747,7 +3772,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C111"/>
+  <dimension ref="A1:C112"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4976,6 +5001,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="112" spans="1:3" ht="16" customHeight="1">
+      <c r="A112" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B112" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C112" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4984,7 +5020,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C111"/>
+  <dimension ref="A1:C112"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6213,6 +6249,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="112" spans="1:3" ht="16" customHeight="1">
+      <c r="A112" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B112" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C112" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6221,7 +6268,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C111"/>
+  <dimension ref="A1:C112"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7450,6 +7497,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="112" spans="1:3" ht="16" customHeight="1">
+      <c r="A112" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B112" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C112" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7458,7 +7516,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C111"/>
+  <dimension ref="A1:C112"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8687,6 +8745,17 @@
         <v>6.79</v>
       </c>
     </row>
+    <row r="112" spans="1:3" ht="16" customHeight="1">
+      <c r="A112" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B112" s="3">
+        <v>6.49</v>
+      </c>
+      <c r="C112" s="3">
+        <v>6.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8695,7 +8764,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C111"/>
+  <dimension ref="A1:C112"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9924,6 +9993,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="112" spans="1:3" ht="16" customHeight="1">
+      <c r="A112" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B112" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C112" s="3">
+        <v>5.44</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9932,7 +10012,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C111"/>
+  <dimension ref="A1:C112"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11161,6 +11241,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="112" spans="1:3" ht="16" customHeight="1">
+      <c r="A112" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B112" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C112" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11169,7 +11260,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C111"/>
+  <dimension ref="A1:C112"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12398,6 +12489,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="112" spans="1:3" ht="16" customHeight="1">
+      <c r="A112" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B112" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C112" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12406,7 +12508,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C111"/>
+  <dimension ref="A1:C112"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13635,6 +13737,17 @@
         <v>3.3453</v>
       </c>
     </row>
+    <row r="112" spans="1:3" ht="16" customHeight="1">
+      <c r="A112" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B112" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C112" s="3">
+        <v>3.49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13643,7 +13756,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C111"/>
+  <dimension ref="A1:C112"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14872,6 +14985,17 @@
         <v>3.1066</v>
       </c>
     </row>
+    <row r="112" spans="1:3" ht="16" customHeight="1">
+      <c r="A112" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B112" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C112" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14880,7 +15004,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C111"/>
+  <dimension ref="A1:C112"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -16109,6 +16233,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="112" spans="1:3" ht="16" customHeight="1">
+      <c r="A112" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B112" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C112" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-29 16:40:17
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3171" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3192" uniqueCount="116">
   <si>
     <t>Date</t>
   </si>
@@ -370,6 +370,9 @@
   </si>
   <si>
     <t>2026-09-28</t>
+  </si>
+  <si>
+    <t>2026-09-29</t>
   </si>
 </sst>
 </file>
@@ -1276,7 +1279,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C112"/>
+  <dimension ref="A1:C113"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2516,6 +2519,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="113" spans="1:3" ht="16" customHeight="1">
+      <c r="A113" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B113" s="3">
+        <v>7.99</v>
+      </c>
+      <c r="C113" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2524,7 +2538,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C112"/>
+  <dimension ref="A1:C113"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3764,6 +3778,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="113" spans="1:3" ht="16" customHeight="1">
+      <c r="A113" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B113" s="3">
+        <v>3.39</v>
+      </c>
+      <c r="C113" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3772,7 +3797,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C112"/>
+  <dimension ref="A1:C113"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5012,6 +5037,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="113" spans="1:3" ht="16" customHeight="1">
+      <c r="A113" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B113" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C113" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5020,7 +5056,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C112"/>
+  <dimension ref="A1:C113"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6260,6 +6296,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="113" spans="1:3" ht="16" customHeight="1">
+      <c r="A113" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B113" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C113" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6268,7 +6315,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C112"/>
+  <dimension ref="A1:C113"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7508,6 +7555,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="113" spans="1:3" ht="16" customHeight="1">
+      <c r="A113" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B113" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C113" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7516,7 +7574,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C112"/>
+  <dimension ref="A1:C113"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8756,6 +8814,17 @@
         <v>6.79</v>
       </c>
     </row>
+    <row r="113" spans="1:3" ht="16" customHeight="1">
+      <c r="A113" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B113" s="3">
+        <v>6.49</v>
+      </c>
+      <c r="C113" s="3">
+        <v>6.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8764,7 +8833,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C112"/>
+  <dimension ref="A1:C113"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10004,6 +10073,17 @@
         <v>5.44</v>
       </c>
     </row>
+    <row r="113" spans="1:3" ht="16" customHeight="1">
+      <c r="A113" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B113" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C113" s="3">
+        <v>5.5333</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10012,7 +10092,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C112"/>
+  <dimension ref="A1:C113"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11252,6 +11332,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="113" spans="1:3" ht="16" customHeight="1">
+      <c r="A113" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B113" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C113" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11260,7 +11351,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C112"/>
+  <dimension ref="A1:C113"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12500,6 +12591,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="113" spans="1:3" ht="16" customHeight="1">
+      <c r="A113" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B113" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C113" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12508,7 +12610,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C112"/>
+  <dimension ref="A1:C113"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13748,6 +13850,17 @@
         <v>3.49</v>
       </c>
     </row>
+    <row r="113" spans="1:3" ht="16" customHeight="1">
+      <c r="A113" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B113" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C113" s="3">
+        <v>3.49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13756,7 +13869,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C112"/>
+  <dimension ref="A1:C113"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14996,6 +15109,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="113" spans="1:3" ht="16" customHeight="1">
+      <c r="A113" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B113" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C113" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -15004,7 +15128,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C112"/>
+  <dimension ref="A1:C113"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -16244,6 +16368,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="113" spans="1:3" ht="16" customHeight="1">
+      <c r="A113" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B113" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C113" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-30 16:32:24
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3192" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3213" uniqueCount="117">
   <si>
     <t>Date</t>
   </si>
@@ -373,6 +373,9 @@
   </si>
   <si>
     <t>2026-09-29</t>
+  </si>
+  <si>
+    <t>2026-09-30</t>
   </si>
 </sst>
 </file>
@@ -1279,7 +1282,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C113"/>
+  <dimension ref="A1:C114"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2530,6 +2533,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="114" spans="1:3" ht="16" customHeight="1">
+      <c r="A114" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B114" s="3">
+        <v>7.99</v>
+      </c>
+      <c r="C114" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2538,7 +2552,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C113"/>
+  <dimension ref="A1:C114"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3789,6 +3803,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="114" spans="1:3" ht="16" customHeight="1">
+      <c r="A114" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B114" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C114" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3797,7 +3822,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C113"/>
+  <dimension ref="A1:C114"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5048,6 +5073,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="114" spans="1:3" ht="16" customHeight="1">
+      <c r="A114" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B114" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C114" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5056,7 +5092,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C113"/>
+  <dimension ref="A1:C114"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6307,6 +6343,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="114" spans="1:3" ht="16" customHeight="1">
+      <c r="A114" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B114" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C114" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6315,7 +6362,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C113"/>
+  <dimension ref="A1:C114"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7566,6 +7613,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="114" spans="1:3" ht="16" customHeight="1">
+      <c r="A114" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B114" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C114" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7574,7 +7632,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C113"/>
+  <dimension ref="A1:C114"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8825,6 +8883,17 @@
         <v>6.79</v>
       </c>
     </row>
+    <row r="114" spans="1:3" ht="16" customHeight="1">
+      <c r="A114" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B114" s="3">
+        <v>7.055</v>
+      </c>
+      <c r="C114" s="3">
+        <v>6.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8833,7 +8902,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C113"/>
+  <dimension ref="A1:C114"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10084,6 +10153,17 @@
         <v>5.5333</v>
       </c>
     </row>
+    <row r="114" spans="1:3" ht="16" customHeight="1">
+      <c r="A114" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B114" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C114" s="3">
+        <v>3.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10092,7 +10172,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C113"/>
+  <dimension ref="A1:C114"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11343,6 +11423,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="114" spans="1:3" ht="16" customHeight="1">
+      <c r="A114" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B114" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C114" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11351,7 +11442,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C113"/>
+  <dimension ref="A1:C114"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12602,6 +12693,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="114" spans="1:3" ht="16" customHeight="1">
+      <c r="A114" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B114" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C114" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12610,7 +12712,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C113"/>
+  <dimension ref="A1:C114"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13861,6 +13963,17 @@
         <v>3.49</v>
       </c>
     </row>
+    <row r="114" spans="1:3" ht="16" customHeight="1">
+      <c r="A114" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B114" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C114" s="3">
+        <v>3.49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13869,7 +13982,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C113"/>
+  <dimension ref="A1:C114"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15120,6 +15233,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="114" spans="1:3" ht="16" customHeight="1">
+      <c r="A114" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B114" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C114" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -15128,7 +15252,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C113"/>
+  <dimension ref="A1:C114"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -16379,6 +16503,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="114" spans="1:3" ht="16" customHeight="1">
+      <c r="A114" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B114" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C114" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-01 17:10:13
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3213" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3235" uniqueCount="118">
   <si>
     <t>Date</t>
   </si>
@@ -376,6 +376,9 @@
   </si>
   <si>
     <t>2026-09-30</t>
+  </si>
+  <si>
+    <t>2026-10-01</t>
   </si>
 </sst>
 </file>
@@ -1282,7 +1285,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C114"/>
+  <dimension ref="A1:C115"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2544,6 +2547,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="115" spans="1:3" ht="16" customHeight="1">
+      <c r="A115" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B115" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C115" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2552,7 +2566,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C114"/>
+  <dimension ref="A1:C115"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3814,6 +3828,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="115" spans="1:3" ht="16" customHeight="1">
+      <c r="A115" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B115" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C115" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3822,7 +3847,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C114"/>
+  <dimension ref="A1:C115"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5084,6 +5109,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="115" spans="1:3" ht="16" customHeight="1">
+      <c r="A115" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B115" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C115" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5092,7 +5128,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C114"/>
+  <dimension ref="A1:C115"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6354,6 +6390,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="115" spans="1:3" ht="16" customHeight="1">
+      <c r="A115" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B115" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C115" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6362,7 +6409,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C114"/>
+  <dimension ref="A1:C115"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7624,6 +7671,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="115" spans="1:3" ht="16" customHeight="1">
+      <c r="A115" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B115" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C115" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7632,7 +7690,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C114"/>
+  <dimension ref="A1:C115"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8894,6 +8952,17 @@
         <v>6.79</v>
       </c>
     </row>
+    <row r="115" spans="1:3" ht="16" customHeight="1">
+      <c r="A115" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B115" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C115" s="3">
+        <v>6.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8902,7 +8971,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C114"/>
+  <dimension ref="A1:C115"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10164,6 +10233,17 @@
         <v>3.79</v>
       </c>
     </row>
+    <row r="115" spans="1:3" ht="16" customHeight="1">
+      <c r="A115" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B115" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C115" s="3">
+        <v>5.5333</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10172,7 +10252,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C114"/>
+  <dimension ref="A1:C115"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11434,6 +11514,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="115" spans="1:3" ht="16" customHeight="1">
+      <c r="A115" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B115" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C115" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11442,7 +11533,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C114"/>
+  <dimension ref="A1:C115"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12704,6 +12795,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="115" spans="1:3" ht="16" customHeight="1">
+      <c r="A115" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B115" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C115" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12712,7 +12814,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C114"/>
+  <dimension ref="A1:C115"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13974,6 +14076,17 @@
         <v>3.49</v>
       </c>
     </row>
+    <row r="115" spans="1:3" ht="16" customHeight="1">
+      <c r="A115" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B115" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C115" s="3">
+        <v>3.49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13982,7 +14095,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C114"/>
+  <dimension ref="A1:C115"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15244,6 +15357,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="115" spans="1:3" ht="16" customHeight="1">
+      <c r="A115" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B115" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C115" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -15252,7 +15376,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C114"/>
+  <dimension ref="A1:C115"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -16514,6 +16638,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="115" spans="1:3" ht="16" customHeight="1">
+      <c r="A115" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B115" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C115" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-02 16:23:38
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3235" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3256" uniqueCount="119">
   <si>
     <t>Date</t>
   </si>
@@ -379,6 +379,9 @@
   </si>
   <si>
     <t>2026-10-01</t>
+  </si>
+  <si>
+    <t>2026-10-02</t>
   </si>
 </sst>
 </file>
@@ -1285,7 +1288,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C115"/>
+  <dimension ref="A1:C116"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2558,6 +2561,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="116" spans="1:3" ht="16" customHeight="1">
+      <c r="A116" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B116" s="3">
+        <v>7.99</v>
+      </c>
+      <c r="C116" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2566,7 +2580,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C115"/>
+  <dimension ref="A1:C116"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3839,6 +3853,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="116" spans="1:3" ht="16" customHeight="1">
+      <c r="A116" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B116" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C116" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3847,7 +3872,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C115"/>
+  <dimension ref="A1:C116"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5120,6 +5145,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="116" spans="1:3" ht="16" customHeight="1">
+      <c r="A116" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B116" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C116" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5128,7 +5164,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C115"/>
+  <dimension ref="A1:C116"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6401,6 +6437,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="116" spans="1:3" ht="16" customHeight="1">
+      <c r="A116" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B116" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C116" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6409,7 +6456,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C115"/>
+  <dimension ref="A1:C116"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7682,6 +7729,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="116" spans="1:3" ht="16" customHeight="1">
+      <c r="A116" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B116" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C116" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7690,7 +7748,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C115"/>
+  <dimension ref="A1:C116"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8963,6 +9021,17 @@
         <v>6.79</v>
       </c>
     </row>
+    <row r="116" spans="1:3" ht="16" customHeight="1">
+      <c r="A116" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B116" s="3">
+        <v>7.125</v>
+      </c>
+      <c r="C116" s="3">
+        <v>6.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8971,7 +9040,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C115"/>
+  <dimension ref="A1:C116"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10244,6 +10313,17 @@
         <v>5.5333</v>
       </c>
     </row>
+    <row r="116" spans="1:3" ht="16" customHeight="1">
+      <c r="A116" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B116" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C116" s="3">
+        <v>5.6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10252,7 +10332,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C115"/>
+  <dimension ref="A1:C116"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11525,6 +11605,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="116" spans="1:3" ht="16" customHeight="1">
+      <c r="A116" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B116" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C116" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11533,7 +11624,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C115"/>
+  <dimension ref="A1:C116"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12806,6 +12897,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="116" spans="1:3" ht="16" customHeight="1">
+      <c r="A116" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B116" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C116" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12814,7 +12916,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C115"/>
+  <dimension ref="A1:C116"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14087,6 +14189,17 @@
         <v>3.49</v>
       </c>
     </row>
+    <row r="116" spans="1:3" ht="16" customHeight="1">
+      <c r="A116" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B116" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C116" s="3">
+        <v>3.49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14095,7 +14208,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C115"/>
+  <dimension ref="A1:C116"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15368,6 +15481,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="116" spans="1:3" ht="16" customHeight="1">
+      <c r="A116" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B116" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C116" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -15376,7 +15500,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C115"/>
+  <dimension ref="A1:C116"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -16649,6 +16773,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="116" spans="1:3" ht="16" customHeight="1">
+      <c r="A116" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B116" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C116" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-03 14:58:39
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3256" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3276" uniqueCount="120">
   <si>
     <t>Date</t>
   </si>
@@ -382,6 +382,9 @@
   </si>
   <si>
     <t>2026-10-02</t>
+  </si>
+  <si>
+    <t>2026-10-03</t>
   </si>
 </sst>
 </file>
@@ -1288,7 +1291,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C116"/>
+  <dimension ref="A1:C117"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2572,6 +2575,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="117" spans="1:3" ht="16" customHeight="1">
+      <c r="A117" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B117" s="3">
+        <v>7.99</v>
+      </c>
+      <c r="C117" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2580,7 +2594,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C116"/>
+  <dimension ref="A1:C117"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3864,6 +3878,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="117" spans="1:3" ht="16" customHeight="1">
+      <c r="A117" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B117" s="3">
+        <v>3.39</v>
+      </c>
+      <c r="C117" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3872,7 +3897,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C116"/>
+  <dimension ref="A1:C117"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5156,6 +5181,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="117" spans="1:3" ht="16" customHeight="1">
+      <c r="A117" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B117" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C117" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5164,7 +5200,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C116"/>
+  <dimension ref="A1:C117"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6448,6 +6484,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="117" spans="1:3" ht="16" customHeight="1">
+      <c r="A117" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B117" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C117" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6456,7 +6503,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C116"/>
+  <dimension ref="A1:C117"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7740,6 +7787,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="117" spans="1:3" ht="16" customHeight="1">
+      <c r="A117" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B117" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C117" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7748,7 +7806,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C116"/>
+  <dimension ref="A1:C117"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9032,6 +9090,17 @@
         <v>6.79</v>
       </c>
     </row>
+    <row r="117" spans="1:3" ht="16" customHeight="1">
+      <c r="A117" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B117" s="3">
+        <v>7.2</v>
+      </c>
+      <c r="C117" s="3">
+        <v>6.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9040,7 +9109,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C116"/>
+  <dimension ref="A1:C117"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10324,6 +10393,17 @@
         <v>5.6</v>
       </c>
     </row>
+    <row r="117" spans="1:3" ht="16" customHeight="1">
+      <c r="A117" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B117" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C117" s="3">
+        <v>3.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10332,7 +10412,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C116"/>
+  <dimension ref="A1:C117"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11616,6 +11696,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="117" spans="1:3" ht="16" customHeight="1">
+      <c r="A117" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B117" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C117" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11624,7 +11715,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C116"/>
+  <dimension ref="A1:C117"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12908,6 +12999,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="117" spans="1:3" ht="16" customHeight="1">
+      <c r="A117" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B117" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C117" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12916,7 +13018,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C116"/>
+  <dimension ref="A1:C117"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14200,6 +14302,17 @@
         <v>3.49</v>
       </c>
     </row>
+    <row r="117" spans="1:3" ht="16" customHeight="1">
+      <c r="A117" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B117" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C117" s="3">
+        <v>3.0134</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14208,7 +14321,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C116"/>
+  <dimension ref="A1:C117"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15492,6 +15605,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="117" spans="1:3" ht="16" customHeight="1">
+      <c r="A117" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B117" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C117" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -15500,7 +15624,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C116"/>
+  <dimension ref="A1:C117"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -16784,6 +16908,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="117" spans="1:3" ht="16" customHeight="1">
+      <c r="A117" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B117" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C117" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-04 15:31:35
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3276" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3296" uniqueCount="121">
   <si>
     <t>Date</t>
   </si>
@@ -385,6 +385,9 @@
   </si>
   <si>
     <t>2026-10-03</t>
+  </si>
+  <si>
+    <t>2026-10-04</t>
   </si>
 </sst>
 </file>
@@ -1291,7 +1294,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C117"/>
+  <dimension ref="A1:C118"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2586,6 +2589,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="118" spans="1:3" ht="16" customHeight="1">
+      <c r="A118" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B118" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C118" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2594,7 +2608,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C117"/>
+  <dimension ref="A1:C118"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3889,6 +3903,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="118" spans="1:3" ht="16" customHeight="1">
+      <c r="A118" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B118" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C118" s="3">
+        <v>2.39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3897,7 +3922,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C117"/>
+  <dimension ref="A1:C118"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5192,6 +5217,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="118" spans="1:3" ht="16" customHeight="1">
+      <c r="A118" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B118" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C118" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5200,7 +5236,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C117"/>
+  <dimension ref="A1:C118"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6495,6 +6531,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="118" spans="1:3" ht="16" customHeight="1">
+      <c r="A118" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B118" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C118" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6503,7 +6550,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C117"/>
+  <dimension ref="A1:C118"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7798,6 +7845,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="118" spans="1:3" ht="16" customHeight="1">
+      <c r="A118" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B118" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C118" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7806,7 +7864,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C117"/>
+  <dimension ref="A1:C118"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9101,6 +9159,17 @@
         <v>6.79</v>
       </c>
     </row>
+    <row r="118" spans="1:3" ht="16" customHeight="1">
+      <c r="A118" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B118" s="3">
+        <v>6.49</v>
+      </c>
+      <c r="C118" s="3">
+        <v>6.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9109,7 +9178,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C117"/>
+  <dimension ref="A1:C118"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10404,6 +10473,17 @@
         <v>3.79</v>
       </c>
     </row>
+    <row r="118" spans="1:3" ht="16" customHeight="1">
+      <c r="A118" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B118" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C118" s="3">
+        <v>3.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10412,7 +10492,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C117"/>
+  <dimension ref="A1:C118"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11707,6 +11787,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="118" spans="1:3" ht="16" customHeight="1">
+      <c r="A118" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B118" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C118" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11715,7 +11806,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C117"/>
+  <dimension ref="A1:C118"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13010,6 +13101,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="118" spans="1:3" ht="16" customHeight="1">
+      <c r="A118" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B118" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C118" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13018,7 +13120,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C117"/>
+  <dimension ref="A1:C118"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14313,6 +14415,17 @@
         <v>3.0134</v>
       </c>
     </row>
+    <row r="118" spans="1:3" ht="16" customHeight="1">
+      <c r="A118" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B118" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C118" s="3">
+        <v>2.8533</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14321,7 +14434,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C117"/>
+  <dimension ref="A1:C118"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15616,6 +15729,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="118" spans="1:3" ht="16" customHeight="1">
+      <c r="A118" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B118" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C118" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -15624,7 +15748,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C117"/>
+  <dimension ref="A1:C118"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -16919,6 +17043,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="118" spans="1:3" ht="16" customHeight="1">
+      <c r="A118" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B118" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C118" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-05 19:30:17
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3296" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3320" uniqueCount="122">
   <si>
     <t>Date</t>
   </si>
@@ -388,6 +388,9 @@
   </si>
   <si>
     <t>2026-10-04</t>
+  </si>
+  <si>
+    <t>2026-10-05</t>
   </si>
 </sst>
 </file>
@@ -1294,7 +1297,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C118"/>
+  <dimension ref="A1:C119"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2600,6 +2603,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="119" spans="1:3" ht="16" customHeight="1">
+      <c r="A119" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B119" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C119" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2608,7 +2622,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C118"/>
+  <dimension ref="A1:C119"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3914,6 +3928,17 @@
         <v>2.39</v>
       </c>
     </row>
+    <row r="119" spans="1:3" ht="16" customHeight="1">
+      <c r="A119" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B119" s="3">
+        <v>3.39</v>
+      </c>
+      <c r="C119" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3922,7 +3947,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C118"/>
+  <dimension ref="A1:C119"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5228,6 +5253,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="119" spans="1:3" ht="16" customHeight="1">
+      <c r="A119" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B119" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C119" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5236,7 +5272,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C118"/>
+  <dimension ref="A1:C119"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6542,6 +6578,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="119" spans="1:3" ht="16" customHeight="1">
+      <c r="A119" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B119" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C119" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6550,7 +6597,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C118"/>
+  <dimension ref="A1:C119"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7856,6 +7903,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="119" spans="1:3" ht="16" customHeight="1">
+      <c r="A119" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B119" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C119" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7864,7 +7922,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C118"/>
+  <dimension ref="A1:C119"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9170,6 +9228,17 @@
         <v>6.79</v>
       </c>
     </row>
+    <row r="119" spans="1:3" ht="16" customHeight="1">
+      <c r="A119" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B119" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C119" s="3">
+        <v>6.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9178,7 +9247,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C118"/>
+  <dimension ref="A1:C119"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10484,6 +10553,17 @@
         <v>3.79</v>
       </c>
     </row>
+    <row r="119" spans="1:3" ht="16" customHeight="1">
+      <c r="A119" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B119" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C119" s="3">
+        <v>4.436</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10492,7 +10572,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C118"/>
+  <dimension ref="A1:C119"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11798,6 +11878,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="119" spans="1:3" ht="16" customHeight="1">
+      <c r="A119" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B119" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C119" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11806,7 +11897,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C118"/>
+  <dimension ref="A1:C119"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13112,6 +13203,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="119" spans="1:3" ht="16" customHeight="1">
+      <c r="A119" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B119" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C119" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13120,7 +13222,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C118"/>
+  <dimension ref="A1:C119"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14426,6 +14528,17 @@
         <v>2.8533</v>
       </c>
     </row>
+    <row r="119" spans="1:3" ht="16" customHeight="1">
+      <c r="A119" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B119" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C119" s="3">
+        <v>2.8253</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14434,7 +14547,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C118"/>
+  <dimension ref="A1:C119"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15740,6 +15853,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="119" spans="1:3" ht="16" customHeight="1">
+      <c r="A119" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B119" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C119" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -15748,7 +15872,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C118"/>
+  <dimension ref="A1:C119"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -17054,6 +17178,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="119" spans="1:3" ht="16" customHeight="1">
+      <c r="A119" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B119" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C119" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-06 16:58:16
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3320" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3342" uniqueCount="123">
   <si>
     <t>Date</t>
   </si>
@@ -391,6 +391,9 @@
   </si>
   <si>
     <t>2026-10-05</t>
+  </si>
+  <si>
+    <t>2026-10-06</t>
   </si>
 </sst>
 </file>
@@ -1297,7 +1300,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C119"/>
+  <dimension ref="A1:C120"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2614,6 +2617,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="120" spans="1:3" ht="16" customHeight="1">
+      <c r="A120" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B120" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C120" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2622,7 +2636,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C119"/>
+  <dimension ref="A1:C120"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3939,6 +3953,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="120" spans="1:3" ht="16" customHeight="1">
+      <c r="A120" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B120" s="3">
+        <v>3.39</v>
+      </c>
+      <c r="C120" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3947,7 +3972,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C119"/>
+  <dimension ref="A1:C120"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5264,6 +5289,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="120" spans="1:3" ht="16" customHeight="1">
+      <c r="A120" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B120" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C120" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5272,7 +5308,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C119"/>
+  <dimension ref="A1:C120"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6589,6 +6625,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="120" spans="1:3" ht="16" customHeight="1">
+      <c r="A120" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B120" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C120" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6597,7 +6644,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C119"/>
+  <dimension ref="A1:C120"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7914,6 +7961,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="120" spans="1:3" ht="16" customHeight="1">
+      <c r="A120" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B120" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C120" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7922,7 +7980,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C119"/>
+  <dimension ref="A1:C120"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9239,6 +9297,17 @@
         <v>6.79</v>
       </c>
     </row>
+    <row r="120" spans="1:3" ht="16" customHeight="1">
+      <c r="A120" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B120" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C120" s="3">
+        <v>6.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9247,7 +9316,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C119"/>
+  <dimension ref="A1:C120"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10564,6 +10633,17 @@
         <v>4.436</v>
       </c>
     </row>
+    <row r="120" spans="1:3" ht="16" customHeight="1">
+      <c r="A120" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B120" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C120" s="3">
+        <v>5.6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10572,7 +10652,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C119"/>
+  <dimension ref="A1:C120"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11889,6 +11969,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="120" spans="1:3" ht="16" customHeight="1">
+      <c r="A120" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B120" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C120" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11897,7 +11988,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C119"/>
+  <dimension ref="A1:C120"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13214,6 +13305,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="120" spans="1:3" ht="16" customHeight="1">
+      <c r="A120" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B120" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C120" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13222,7 +13324,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C119"/>
+  <dimension ref="A1:C120"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14539,6 +14641,17 @@
         <v>2.8253</v>
       </c>
     </row>
+    <row r="120" spans="1:3" ht="16" customHeight="1">
+      <c r="A120" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B120" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C120" s="3">
+        <v>3.1854</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14547,7 +14660,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C119"/>
+  <dimension ref="A1:C120"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15864,6 +15977,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="120" spans="1:3" ht="16" customHeight="1">
+      <c r="A120" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B120" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C120" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -15872,7 +15996,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C119"/>
+  <dimension ref="A1:C120"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -17189,6 +17313,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="120" spans="1:3" ht="16" customHeight="1">
+      <c r="A120" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B120" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C120" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-07 17:34:24
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3342" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3365" uniqueCount="124">
   <si>
     <t>Date</t>
   </si>
@@ -395,6 +395,9 @@
   <si>
     <t>2026-10-06</t>
   </si>
+  <si>
+    <t>2026-10-07</t>
+  </si>
 </sst>
 </file>
 
@@ -510,7 +513,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -530,7 +533,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -553,7 +556,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -573,7 +576,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -596,7 +599,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -616,7 +619,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -639,7 +642,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -659,7 +662,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -725,7 +728,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -745,7 +748,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -768,7 +771,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -788,7 +791,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -811,7 +814,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -831,7 +834,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -854,7 +857,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -874,7 +877,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -897,7 +900,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -917,7 +920,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -940,7 +943,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -960,7 +963,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1300,7 +1303,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C120"/>
+  <dimension ref="A1:C121"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2628,6 +2631,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="121" spans="1:3" ht="16" customHeight="1">
+      <c r="A121" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B121" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C121" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2636,7 +2650,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C120"/>
+  <dimension ref="A1:C121"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3964,6 +3978,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="121" spans="1:3" ht="16" customHeight="1">
+      <c r="A121" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B121" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C121" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3972,7 +3997,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C120"/>
+  <dimension ref="A1:C121"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5300,6 +5325,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="121" spans="1:3" ht="16" customHeight="1">
+      <c r="A121" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B121" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C121" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5308,7 +5344,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C120"/>
+  <dimension ref="A1:C121"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6636,6 +6672,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="121" spans="1:3" ht="16" customHeight="1">
+      <c r="A121" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B121" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C121" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6644,7 +6691,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C120"/>
+  <dimension ref="A1:C121"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7972,6 +8019,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="121" spans="1:3" ht="16" customHeight="1">
+      <c r="A121" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B121" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C121" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7980,7 +8038,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C120"/>
+  <dimension ref="A1:C121"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9308,6 +9366,17 @@
         <v>6.79</v>
       </c>
     </row>
+    <row r="121" spans="1:3" ht="16" customHeight="1">
+      <c r="A121" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B121" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C121" s="3">
+        <v>6.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9316,7 +9385,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C120"/>
+  <dimension ref="A1:C121"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10644,6 +10713,17 @@
         <v>5.6</v>
       </c>
     </row>
+    <row r="121" spans="1:3" ht="16" customHeight="1">
+      <c r="A121" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B121" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C121" s="3">
+        <v>5.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10652,7 +10732,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C120"/>
+  <dimension ref="A1:C121"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11980,6 +12060,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="121" spans="1:3" ht="16" customHeight="1">
+      <c r="A121" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B121" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C121" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11988,7 +12079,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C120"/>
+  <dimension ref="A1:C121"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13316,6 +13407,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="121" spans="1:3" ht="16" customHeight="1">
+      <c r="A121" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B121" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C121" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13324,7 +13426,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C120"/>
+  <dimension ref="A1:C121"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14652,6 +14754,17 @@
         <v>3.1854</v>
       </c>
     </row>
+    <row r="121" spans="1:3" ht="16" customHeight="1">
+      <c r="A121" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B121" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C121" s="3">
+        <v>3.49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14660,7 +14773,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C120"/>
+  <dimension ref="A1:C121"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15988,6 +16101,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="121" spans="1:3" ht="16" customHeight="1">
+      <c r="A121" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B121" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C121" s="3">
+        <v>3.1707</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -15996,7 +16120,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C120"/>
+  <dimension ref="A1:C121"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -17324,6 +17448,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="121" spans="1:3" ht="16" customHeight="1">
+      <c r="A121" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B121" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C121" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-08 17:37:43
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3365" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3388" uniqueCount="125">
   <si>
     <t>Date</t>
   </si>
@@ -398,6 +398,9 @@
   <si>
     <t>2026-10-07</t>
   </si>
+  <si>
+    <t>2026-10-08</t>
+  </si>
 </sst>
 </file>
 
@@ -513,7 +516,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -533,7 +536,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -556,7 +559,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -576,7 +579,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -599,7 +602,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -619,7 +622,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -642,7 +645,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -662,7 +665,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -728,7 +731,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -748,7 +751,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -771,7 +774,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -791,7 +794,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -814,7 +817,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -834,7 +837,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -857,7 +860,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -877,7 +880,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -900,7 +903,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -920,7 +923,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -943,7 +946,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -963,7 +966,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1303,7 +1306,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C121"/>
+  <dimension ref="A1:C122"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2642,6 +2645,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="122" spans="1:3" ht="16" customHeight="1">
+      <c r="A122" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B122" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C122" s="3">
+        <v>8.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2650,7 +2664,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C121"/>
+  <dimension ref="A1:C122"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3989,6 +4003,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="122" spans="1:3" ht="16" customHeight="1">
+      <c r="A122" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B122" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C122" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3997,7 +4022,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C121"/>
+  <dimension ref="A1:C122"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5336,6 +5361,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="122" spans="1:3" ht="16" customHeight="1">
+      <c r="A122" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B122" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C122" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5344,7 +5380,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C121"/>
+  <dimension ref="A1:C122"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6683,6 +6719,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="122" spans="1:3" ht="16" customHeight="1">
+      <c r="A122" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B122" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C122" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6691,7 +6738,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C121"/>
+  <dimension ref="A1:C122"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8030,6 +8077,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="122" spans="1:3" ht="16" customHeight="1">
+      <c r="A122" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B122" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C122" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8038,7 +8096,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C121"/>
+  <dimension ref="A1:C122"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9377,6 +9435,17 @@
         <v>6.79</v>
       </c>
     </row>
+    <row r="122" spans="1:3" ht="16" customHeight="1">
+      <c r="A122" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B122" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C122" s="3">
+        <v>7.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9385,7 +9454,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C121"/>
+  <dimension ref="A1:C122"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10724,6 +10793,17 @@
         <v>5.5</v>
       </c>
     </row>
+    <row r="122" spans="1:3" ht="16" customHeight="1">
+      <c r="A122" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B122" s="3">
+        <v>3.59</v>
+      </c>
+      <c r="C122" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10732,7 +10812,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C121"/>
+  <dimension ref="A1:C122"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12071,6 +12151,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="122" spans="1:3" ht="16" customHeight="1">
+      <c r="A122" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B122" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C122" s="3">
+        <v>5.29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12079,7 +12170,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C121"/>
+  <dimension ref="A1:C122"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13418,6 +13509,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="122" spans="1:3" ht="16" customHeight="1">
+      <c r="A122" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B122" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C122" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13426,7 +13528,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C121"/>
+  <dimension ref="A1:C122"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14765,6 +14867,17 @@
         <v>3.49</v>
       </c>
     </row>
+    <row r="122" spans="1:3" ht="16" customHeight="1">
+      <c r="A122" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B122" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C122" s="3">
+        <v>3.5853</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14773,7 +14886,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C121"/>
+  <dimension ref="A1:C122"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -16112,6 +16225,17 @@
         <v>3.1707</v>
       </c>
     </row>
+    <row r="122" spans="1:3" ht="16" customHeight="1">
+      <c r="A122" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B122" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C122" s="3">
+        <v>3.4907</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -16120,7 +16244,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C121"/>
+  <dimension ref="A1:C122"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -17459,6 +17583,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="122" spans="1:3" ht="16" customHeight="1">
+      <c r="A122" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B122" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C122" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-09 17:13:38
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3388" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3411" uniqueCount="126">
   <si>
     <t>Date</t>
   </si>
@@ -401,6 +401,9 @@
   <si>
     <t>2026-10-08</t>
   </si>
+  <si>
+    <t>2026-10-09</t>
+  </si>
 </sst>
 </file>
 
@@ -516,7 +519,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -536,7 +539,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -559,7 +562,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -579,7 +582,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -602,7 +605,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -622,7 +625,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -645,7 +648,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -665,7 +668,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -731,7 +734,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -751,7 +754,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -774,7 +777,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -794,7 +797,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -817,7 +820,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -837,7 +840,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -860,7 +863,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -880,7 +883,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -903,7 +906,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -923,7 +926,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -946,7 +949,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -966,7 +969,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1306,7 +1309,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C122"/>
+  <dimension ref="A1:C123"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2656,6 +2659,17 @@
         <v>8.99</v>
       </c>
     </row>
+    <row r="123" spans="1:3" ht="16" customHeight="1">
+      <c r="A123" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B123" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C123" s="3">
+        <v>8.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2664,7 +2678,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C122"/>
+  <dimension ref="A1:C123"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4014,6 +4028,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="123" spans="1:3" ht="16" customHeight="1">
+      <c r="A123" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B123" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C123" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4022,7 +4047,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C122"/>
+  <dimension ref="A1:C123"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5372,6 +5397,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="123" spans="1:3" ht="16" customHeight="1">
+      <c r="A123" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B123" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C123" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5380,7 +5416,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C122"/>
+  <dimension ref="A1:C123"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6730,6 +6766,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="123" spans="1:3" ht="16" customHeight="1">
+      <c r="A123" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B123" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C123" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6738,7 +6785,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C122"/>
+  <dimension ref="A1:C123"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8088,6 +8135,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="123" spans="1:3" ht="16" customHeight="1">
+      <c r="A123" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B123" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C123" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8096,7 +8154,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C122"/>
+  <dimension ref="A1:C123"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9446,6 +9504,17 @@
         <v>7.5</v>
       </c>
     </row>
+    <row r="123" spans="1:3" ht="16" customHeight="1">
+      <c r="A123" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B123" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C123" s="3">
+        <v>7.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9454,7 +9523,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C122"/>
+  <dimension ref="A1:C123"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10804,6 +10873,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="123" spans="1:3" ht="16" customHeight="1">
+      <c r="A123" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B123" s="3">
+        <v>3.59</v>
+      </c>
+      <c r="C123" s="3">
+        <v>10.6667</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10812,7 +10892,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C122"/>
+  <dimension ref="A1:C123"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12162,6 +12242,17 @@
         <v>5.29</v>
       </c>
     </row>
+    <row r="123" spans="1:3" ht="16" customHeight="1">
+      <c r="A123" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B123" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C123" s="3">
+        <v>5.29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12170,7 +12261,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C122"/>
+  <dimension ref="A1:C123"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13520,6 +13611,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="123" spans="1:3" ht="16" customHeight="1">
+      <c r="A123" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B123" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C123" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13528,7 +13630,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C122"/>
+  <dimension ref="A1:C123"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14878,6 +14980,17 @@
         <v>3.5853</v>
       </c>
     </row>
+    <row r="123" spans="1:3" ht="16" customHeight="1">
+      <c r="A123" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B123" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C123" s="3">
+        <v>3.1453</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14886,7 +14999,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C122"/>
+  <dimension ref="A1:C123"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -16236,6 +16349,17 @@
         <v>3.4907</v>
       </c>
     </row>
+    <row r="123" spans="1:3" ht="16" customHeight="1">
+      <c r="A123" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B123" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C123" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -16244,7 +16368,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C122"/>
+  <dimension ref="A1:C123"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -17594,6 +17718,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="123" spans="1:3" ht="16" customHeight="1">
+      <c r="A123" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B123" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C123" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-10 15:58:20
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3411" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3433" uniqueCount="127">
   <si>
     <t>Date</t>
   </si>
@@ -404,6 +404,9 @@
   <si>
     <t>2026-10-09</t>
   </si>
+  <si>
+    <t>2026-10-10</t>
+  </si>
 </sst>
 </file>
 
@@ -519,7 +522,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -539,7 +542,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -562,7 +565,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -582,7 +585,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -605,7 +608,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -625,7 +628,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -648,7 +651,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -668,7 +671,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -734,7 +737,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -754,7 +757,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -820,7 +823,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -840,7 +843,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -863,7 +866,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -883,7 +886,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -906,7 +909,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -926,7 +929,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -949,7 +952,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -969,7 +972,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1309,7 +1312,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C123"/>
+  <dimension ref="A1:C124"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2670,6 +2673,17 @@
         <v>8.99</v>
       </c>
     </row>
+    <row r="124" spans="1:3" ht="16" customHeight="1">
+      <c r="A124" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B124" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C124" s="3">
+        <v>8.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2678,7 +2692,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C123"/>
+  <dimension ref="A1:C124"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4039,6 +4053,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="124" spans="1:3" ht="16" customHeight="1">
+      <c r="A124" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B124" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C124" s="3">
+        <v>2.39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4047,7 +4072,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C123"/>
+  <dimension ref="A1:C124"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5408,6 +5433,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="124" spans="1:3" ht="16" customHeight="1">
+      <c r="A124" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B124" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C124" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5416,7 +5452,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C123"/>
+  <dimension ref="A1:C124"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6777,6 +6813,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="124" spans="1:3" ht="16" customHeight="1">
+      <c r="A124" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B124" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C124" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6785,7 +6832,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C123"/>
+  <dimension ref="A1:C124"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8146,6 +8193,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="124" spans="1:3" ht="16" customHeight="1">
+      <c r="A124" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B124" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C124" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8154,7 +8212,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C123"/>
+  <dimension ref="A1:C124"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9515,6 +9573,17 @@
         <v>7.5</v>
       </c>
     </row>
+    <row r="124" spans="1:3" ht="16" customHeight="1">
+      <c r="A124" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B124" s="3">
+        <v>6.49</v>
+      </c>
+      <c r="C124" s="3">
+        <v>7.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9523,7 +9592,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C123"/>
+  <dimension ref="A1:C124"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10884,6 +10953,17 @@
         <v>10.6667</v>
       </c>
     </row>
+    <row r="124" spans="1:3" ht="16" customHeight="1">
+      <c r="A124" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B124" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C124" s="3">
+        <v>5.84</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10892,7 +10972,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C123"/>
+  <dimension ref="A1:C124"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12253,6 +12333,17 @@
         <v>5.29</v>
       </c>
     </row>
+    <row r="124" spans="1:3" ht="16" customHeight="1">
+      <c r="A124" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B124" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C124" s="3">
+        <v>5.29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12261,7 +12352,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C123"/>
+  <dimension ref="A1:C124"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13622,6 +13713,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="124" spans="1:3" ht="16" customHeight="1">
+      <c r="A124" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B124" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C124" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13630,7 +13732,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C123"/>
+  <dimension ref="A1:C124"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14991,6 +15093,17 @@
         <v>3.1453</v>
       </c>
     </row>
+    <row r="124" spans="1:3" ht="16" customHeight="1">
+      <c r="A124" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B124" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C124" s="3">
+        <v>3.7306</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14999,7 +15112,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C123"/>
+  <dimension ref="A1:C124"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -16360,6 +16473,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="124" spans="1:3" ht="16" customHeight="1">
+      <c r="A124" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B124" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C124" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -16368,7 +16492,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C123"/>
+  <dimension ref="A1:C124"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -17729,6 +17853,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="124" spans="1:3" ht="16" customHeight="1">
+      <c r="A124" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B124" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C124" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-11 16:26:32
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3433" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3455" uniqueCount="128">
   <si>
     <t>Date</t>
   </si>
@@ -406,6 +406,9 @@
   </si>
   <si>
     <t>2026-10-10</t>
+  </si>
+  <si>
+    <t>2026-10-11</t>
   </si>
 </sst>
 </file>
@@ -1312,7 +1315,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C124"/>
+  <dimension ref="A1:C125"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2684,6 +2687,17 @@
         <v>8.99</v>
       </c>
     </row>
+    <row r="125" spans="1:3" ht="16" customHeight="1">
+      <c r="A125" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B125" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C125" s="3">
+        <v>8.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2692,7 +2706,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C124"/>
+  <dimension ref="A1:C125"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4064,6 +4078,17 @@
         <v>2.39</v>
       </c>
     </row>
+    <row r="125" spans="1:3" ht="16" customHeight="1">
+      <c r="A125" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B125" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C125" s="3">
+        <v>2.39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4072,7 +4097,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C124"/>
+  <dimension ref="A1:C125"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5444,6 +5469,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="125" spans="1:3" ht="16" customHeight="1">
+      <c r="A125" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B125" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C125" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5452,7 +5488,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C124"/>
+  <dimension ref="A1:C125"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6824,6 +6860,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="125" spans="1:3" ht="16" customHeight="1">
+      <c r="A125" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B125" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C125" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6832,7 +6879,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C124"/>
+  <dimension ref="A1:C125"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8204,6 +8251,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="125" spans="1:3" ht="16" customHeight="1">
+      <c r="A125" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B125" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C125" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8212,7 +8270,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C124"/>
+  <dimension ref="A1:C125"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9584,6 +9642,17 @@
         <v>7.5</v>
       </c>
     </row>
+    <row r="125" spans="1:3" ht="16" customHeight="1">
+      <c r="A125" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B125" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C125" s="3">
+        <v>7.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9592,7 +9661,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C124"/>
+  <dimension ref="A1:C125"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10964,6 +11033,17 @@
         <v>5.84</v>
       </c>
     </row>
+    <row r="125" spans="1:3" ht="16" customHeight="1">
+      <c r="A125" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B125" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C125" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10972,7 +11052,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C124"/>
+  <dimension ref="A1:C125"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12344,6 +12424,17 @@
         <v>5.29</v>
       </c>
     </row>
+    <row r="125" spans="1:3" ht="16" customHeight="1">
+      <c r="A125" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B125" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C125" s="3">
+        <v>5.29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12352,7 +12443,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C124"/>
+  <dimension ref="A1:C125"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13724,6 +13815,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="125" spans="1:3" ht="16" customHeight="1">
+      <c r="A125" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B125" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C125" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13732,7 +13834,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C124"/>
+  <dimension ref="A1:C125"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15104,6 +15206,17 @@
         <v>3.7306</v>
       </c>
     </row>
+    <row r="125" spans="1:3" ht="16" customHeight="1">
+      <c r="A125" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B125" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C125" s="3">
+        <v>3.6253</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -15112,7 +15225,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C124"/>
+  <dimension ref="A1:C125"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -16484,6 +16597,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="125" spans="1:3" ht="16" customHeight="1">
+      <c r="A125" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B125" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C125" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -16492,7 +16616,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C124"/>
+  <dimension ref="A1:C125"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -17864,6 +17988,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="125" spans="1:3" ht="16" customHeight="1">
+      <c r="A125" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B125" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C125" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-12 20:01:30
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3455" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3475" uniqueCount="129">
   <si>
     <t>Date</t>
   </si>
@@ -409,6 +409,9 @@
   </si>
   <si>
     <t>2026-10-11</t>
+  </si>
+  <si>
+    <t>2026-10-12</t>
   </si>
 </sst>
 </file>
@@ -1315,7 +1318,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C125"/>
+  <dimension ref="A1:C126"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2698,6 +2701,17 @@
         <v>8.99</v>
       </c>
     </row>
+    <row r="126" spans="1:3" ht="16" customHeight="1">
+      <c r="A126" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B126" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C126" s="3">
+        <v>8.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2706,7 +2720,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C125"/>
+  <dimension ref="A1:C126"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4089,6 +4103,17 @@
         <v>2.39</v>
       </c>
     </row>
+    <row r="126" spans="1:3" ht="16" customHeight="1">
+      <c r="A126" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B126" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C126" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4097,7 +4122,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C125"/>
+  <dimension ref="A1:C126"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5480,6 +5505,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="126" spans="1:3" ht="16" customHeight="1">
+      <c r="A126" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B126" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C126" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5488,7 +5524,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C125"/>
+  <dimension ref="A1:C126"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6871,6 +6907,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="126" spans="1:3" ht="16" customHeight="1">
+      <c r="A126" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B126" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C126" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6879,7 +6926,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C125"/>
+  <dimension ref="A1:C126"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8262,6 +8309,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="126" spans="1:3" ht="16" customHeight="1">
+      <c r="A126" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B126" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C126" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8270,7 +8328,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C125"/>
+  <dimension ref="A1:C126"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9653,6 +9711,17 @@
         <v>7.5</v>
       </c>
     </row>
+    <row r="126" spans="1:3" ht="16" customHeight="1">
+      <c r="A126" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B126" s="3">
+        <v>7.7925</v>
+      </c>
+      <c r="C126" s="3">
+        <v>7.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9661,7 +9730,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C125"/>
+  <dimension ref="A1:C126"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11044,6 +11113,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="126" spans="1:3" ht="16" customHeight="1">
+      <c r="A126" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B126" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C126" s="3">
+        <v>5.96</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11052,7 +11132,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C125"/>
+  <dimension ref="A1:C126"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12435,6 +12515,17 @@
         <v>5.29</v>
       </c>
     </row>
+    <row r="126" spans="1:3" ht="16" customHeight="1">
+      <c r="A126" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B126" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C126" s="3">
+        <v>5.29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12443,7 +12534,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C125"/>
+  <dimension ref="A1:C126"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13826,6 +13917,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="126" spans="1:3" ht="16" customHeight="1">
+      <c r="A126" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B126" s="3">
+        <v>1.99</v>
+      </c>
+      <c r="C126" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13834,7 +13936,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C125"/>
+  <dimension ref="A1:C126"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15217,6 +15319,17 @@
         <v>3.6253</v>
       </c>
     </row>
+    <row r="126" spans="1:3" ht="16" customHeight="1">
+      <c r="A126" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B126" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C126" s="3">
+        <v>3.3853</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -15225,7 +15338,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C125"/>
+  <dimension ref="A1:C126"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -16608,6 +16721,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="126" spans="1:3" ht="16" customHeight="1">
+      <c r="A126" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B126" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C126" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -16616,7 +16740,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C125"/>
+  <dimension ref="A1:C126"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -17999,6 +18123,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="126" spans="1:3" ht="16" customHeight="1">
+      <c r="A126" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B126" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C126" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-13 17:50:09
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3475" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3499" uniqueCount="130">
   <si>
     <t>Date</t>
   </si>
@@ -412,6 +412,9 @@
   </si>
   <si>
     <t>2026-10-12</t>
+  </si>
+  <si>
+    <t>2026-10-13</t>
   </si>
 </sst>
 </file>
@@ -1318,7 +1321,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C126"/>
+  <dimension ref="A1:C127"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2712,6 +2715,17 @@
         <v>8.99</v>
       </c>
     </row>
+    <row r="127" spans="1:3" ht="16" customHeight="1">
+      <c r="A127" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B127" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C127" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2720,7 +2734,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C126"/>
+  <dimension ref="A1:C127"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4114,6 +4128,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="127" spans="1:3" ht="16" customHeight="1">
+      <c r="A127" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B127" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C127" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4122,7 +4147,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C126"/>
+  <dimension ref="A1:C127"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5516,6 +5541,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="127" spans="1:3" ht="16" customHeight="1">
+      <c r="A127" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B127" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C127" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5524,7 +5560,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C126"/>
+  <dimension ref="A1:C127"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6918,6 +6954,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="127" spans="1:3" ht="16" customHeight="1">
+      <c r="A127" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B127" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C127" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6926,7 +6973,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C126"/>
+  <dimension ref="A1:C127"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8320,6 +8367,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="127" spans="1:3" ht="16" customHeight="1">
+      <c r="A127" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B127" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C127" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8328,7 +8386,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C126"/>
+  <dimension ref="A1:C127"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9722,6 +9780,17 @@
         <v>7.5</v>
       </c>
     </row>
+    <row r="127" spans="1:3" ht="16" customHeight="1">
+      <c r="A127" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B127" s="3">
+        <v>7.87</v>
+      </c>
+      <c r="C127" s="3">
+        <v>7.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9730,7 +9799,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C126"/>
+  <dimension ref="A1:C127"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11124,6 +11193,17 @@
         <v>5.96</v>
       </c>
     </row>
+    <row r="127" spans="1:3" ht="16" customHeight="1">
+      <c r="A127" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B127" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C127" s="3">
+        <v>3.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11132,7 +11212,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C126"/>
+  <dimension ref="A1:C127"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12526,6 +12606,17 @@
         <v>5.29</v>
       </c>
     </row>
+    <row r="127" spans="1:3" ht="16" customHeight="1">
+      <c r="A127" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B127" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C127" s="3">
+        <v>5.29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12534,7 +12625,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C126"/>
+  <dimension ref="A1:C127"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13928,6 +14019,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="127" spans="1:3" ht="16" customHeight="1">
+      <c r="A127" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B127" s="3">
+        <v>1.99</v>
+      </c>
+      <c r="C127" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13936,7 +14038,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C126"/>
+  <dimension ref="A1:C127"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15330,6 +15432,17 @@
         <v>3.3853</v>
       </c>
     </row>
+    <row r="127" spans="1:3" ht="16" customHeight="1">
+      <c r="A127" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B127" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C127" s="3">
+        <v>3.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -15338,7 +15451,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C126"/>
+  <dimension ref="A1:C127"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -16732,6 +16845,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="127" spans="1:3" ht="16" customHeight="1">
+      <c r="A127" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B127" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C127" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -16740,7 +16864,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C126"/>
+  <dimension ref="A1:C127"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -18134,6 +18258,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="127" spans="1:3" ht="16" customHeight="1">
+      <c r="A127" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B127" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C127" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-14 15:34:48
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3499" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3521" uniqueCount="131">
   <si>
     <t>Date</t>
   </si>
@@ -415,6 +415,9 @@
   </si>
   <si>
     <t>2026-10-13</t>
+  </si>
+  <si>
+    <t>2026-10-14</t>
   </si>
 </sst>
 </file>
@@ -1321,7 +1324,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C127"/>
+  <dimension ref="A1:C128"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2726,6 +2729,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="128" spans="1:3" ht="16" customHeight="1">
+      <c r="A128" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B128" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C128" s="3">
+        <v>8.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2734,7 +2748,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C127"/>
+  <dimension ref="A1:C128"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4139,6 +4153,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="128" spans="1:3" ht="16" customHeight="1">
+      <c r="A128" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B128" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C128" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4147,7 +4172,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C127"/>
+  <dimension ref="A1:C128"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5552,6 +5577,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="128" spans="1:3" ht="16" customHeight="1">
+      <c r="A128" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B128" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C128" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5560,7 +5596,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C127"/>
+  <dimension ref="A1:C128"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6965,6 +7001,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="128" spans="1:3" ht="16" customHeight="1">
+      <c r="A128" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B128" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C128" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6973,7 +7020,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C127"/>
+  <dimension ref="A1:C128"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8378,6 +8425,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="128" spans="1:3" ht="16" customHeight="1">
+      <c r="A128" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B128" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C128" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8386,7 +8444,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C127"/>
+  <dimension ref="A1:C128"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9791,6 +9849,17 @@
         <v>7.99</v>
       </c>
     </row>
+    <row r="128" spans="1:3" ht="16" customHeight="1">
+      <c r="A128" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B128" s="3">
+        <v>7.95</v>
+      </c>
+      <c r="C128" s="3">
+        <v>7.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9799,7 +9868,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C127"/>
+  <dimension ref="A1:C128"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11204,6 +11273,17 @@
         <v>3.79</v>
       </c>
     </row>
+    <row r="128" spans="1:3" ht="16" customHeight="1">
+      <c r="A128" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B128" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C128" s="3">
+        <v>3.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11212,7 +11292,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C127"/>
+  <dimension ref="A1:C128"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12617,6 +12697,17 @@
         <v>5.29</v>
       </c>
     </row>
+    <row r="128" spans="1:3" ht="16" customHeight="1">
+      <c r="A128" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B128" s="3">
+        <v>4.29</v>
+      </c>
+      <c r="C128" s="3">
+        <v>5.29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12625,7 +12716,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C127"/>
+  <dimension ref="A1:C128"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14030,6 +14121,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="128" spans="1:3" ht="16" customHeight="1">
+      <c r="A128" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B128" s="3">
+        <v>1.99</v>
+      </c>
+      <c r="C128" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14038,7 +14140,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C127"/>
+  <dimension ref="A1:C128"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15443,6 +15545,17 @@
         <v>3.99</v>
       </c>
     </row>
+    <row r="128" spans="1:3" ht="16" customHeight="1">
+      <c r="A128" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B128" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C128" s="3">
+        <v>3.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -15451,7 +15564,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C127"/>
+  <dimension ref="A1:C128"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -16856,6 +16969,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="128" spans="1:3" ht="16" customHeight="1">
+      <c r="A128" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B128" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C128" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -16864,7 +16988,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C127"/>
+  <dimension ref="A1:C128"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -18269,6 +18393,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="128" spans="1:3" ht="16" customHeight="1">
+      <c r="A128" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B128" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C128" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-15 15:22:40
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3521" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3542" uniqueCount="132">
   <si>
     <t>Date</t>
   </si>
@@ -418,6 +418,9 @@
   </si>
   <si>
     <t>2026-10-14</t>
+  </si>
+  <si>
+    <t>2026-10-15</t>
   </si>
 </sst>
 </file>
@@ -1324,7 +1327,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C128"/>
+  <dimension ref="A1:C129"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2740,6 +2743,17 @@
         <v>8.99</v>
       </c>
     </row>
+    <row r="129" spans="1:3" ht="16" customHeight="1">
+      <c r="A129" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B129" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C129" s="3">
+        <v>8.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2748,7 +2762,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C128"/>
+  <dimension ref="A1:C129"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4164,6 +4178,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="129" spans="1:3" ht="16" customHeight="1">
+      <c r="A129" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B129" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C129" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4172,7 +4197,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C128"/>
+  <dimension ref="A1:C129"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5588,6 +5613,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="129" spans="1:3" ht="16" customHeight="1">
+      <c r="A129" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B129" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C129" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5596,7 +5632,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C128"/>
+  <dimension ref="A1:C129"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7012,6 +7048,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="129" spans="1:3" ht="16" customHeight="1">
+      <c r="A129" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B129" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C129" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7020,7 +7067,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C128"/>
+  <dimension ref="A1:C129"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8436,6 +8483,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="129" spans="1:3" ht="16" customHeight="1">
+      <c r="A129" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B129" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C129" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8444,7 +8502,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C128"/>
+  <dimension ref="A1:C129"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9860,6 +9918,17 @@
         <v>7.99</v>
       </c>
     </row>
+    <row r="129" spans="1:3" ht="16" customHeight="1">
+      <c r="A129" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B129" s="3">
+        <v>8.0288</v>
+      </c>
+      <c r="C129" s="3">
+        <v>7.875</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9868,7 +9937,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C128"/>
+  <dimension ref="A1:C129"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11284,6 +11353,17 @@
         <v>3.79</v>
       </c>
     </row>
+    <row r="129" spans="1:3" ht="16" customHeight="1">
+      <c r="A129" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B129" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C129" s="3">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11292,7 +11372,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C128"/>
+  <dimension ref="A1:C129"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12708,6 +12788,17 @@
         <v>5.29</v>
       </c>
     </row>
+    <row r="129" spans="1:3" ht="16" customHeight="1">
+      <c r="A129" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B129" s="3">
+        <v>4.29</v>
+      </c>
+      <c r="C129" s="3">
+        <v>5.29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12716,7 +12807,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C128"/>
+  <dimension ref="A1:C129"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14132,6 +14223,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="129" spans="1:3" ht="16" customHeight="1">
+      <c r="A129" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B129" s="3">
+        <v>1.99</v>
+      </c>
+      <c r="C129" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14140,7 +14242,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C128"/>
+  <dimension ref="A1:C129"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15556,6 +15658,17 @@
         <v>3.99</v>
       </c>
     </row>
+    <row r="129" spans="1:3" ht="16" customHeight="1">
+      <c r="A129" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B129" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C129" s="3">
+        <v>3.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -15564,7 +15677,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C128"/>
+  <dimension ref="A1:C129"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -16980,6 +17093,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="129" spans="1:3" ht="16" customHeight="1">
+      <c r="A129" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B129" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C129" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -16988,7 +17112,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C128"/>
+  <dimension ref="A1:C129"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -18404,6 +18528,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="129" spans="1:3" ht="16" customHeight="1">
+      <c r="A129" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B129" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C129" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-16 15:03:01
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3542" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3563" uniqueCount="133">
   <si>
     <t>Date</t>
   </si>
@@ -421,6 +421,9 @@
   </si>
   <si>
     <t>2026-10-15</t>
+  </si>
+  <si>
+    <t>2026-10-16</t>
   </si>
 </sst>
 </file>
@@ -1327,7 +1330,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C129"/>
+  <dimension ref="A1:C130"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2754,6 +2757,17 @@
         <v>8.99</v>
       </c>
     </row>
+    <row r="130" spans="1:3" ht="16" customHeight="1">
+      <c r="A130" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B130" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C130" s="3">
+        <v>8.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2762,7 +2776,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C129"/>
+  <dimension ref="A1:C130"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4189,6 +4203,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="130" spans="1:3" ht="16" customHeight="1">
+      <c r="A130" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B130" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C130" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4197,7 +4222,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C129"/>
+  <dimension ref="A1:C130"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5624,6 +5649,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="130" spans="1:3" ht="16" customHeight="1">
+      <c r="A130" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B130" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C130" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5632,7 +5668,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C129"/>
+  <dimension ref="A1:C130"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7059,6 +7095,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="130" spans="1:3" ht="16" customHeight="1">
+      <c r="A130" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B130" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C130" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7067,7 +7114,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C129"/>
+  <dimension ref="A1:C130"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8494,6 +8541,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="130" spans="1:3" ht="16" customHeight="1">
+      <c r="A130" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B130" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C130" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8502,7 +8560,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C129"/>
+  <dimension ref="A1:C130"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9929,6 +9987,17 @@
         <v>7.875</v>
       </c>
     </row>
+    <row r="130" spans="1:3" ht="16" customHeight="1">
+      <c r="A130" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B130" s="3">
+        <v>8.0688</v>
+      </c>
+      <c r="C130" s="3">
+        <v>7.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9937,7 +10006,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C129"/>
+  <dimension ref="A1:C130"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11364,6 +11433,17 @@
         <v>6</v>
       </c>
     </row>
+    <row r="130" spans="1:3" ht="16" customHeight="1">
+      <c r="A130" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B130" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C130" s="3">
+        <v>3.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11372,7 +11452,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C129"/>
+  <dimension ref="A1:C130"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12799,6 +12879,17 @@
         <v>5.29</v>
       </c>
     </row>
+    <row r="130" spans="1:3" ht="16" customHeight="1">
+      <c r="A130" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B130" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C130" s="3">
+        <v>5.29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12807,7 +12898,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C129"/>
+  <dimension ref="A1:C130"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14234,6 +14325,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="130" spans="1:3" ht="16" customHeight="1">
+      <c r="A130" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B130" s="3">
+        <v>1.99</v>
+      </c>
+      <c r="C130" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14242,7 +14344,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C129"/>
+  <dimension ref="A1:C130"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15669,6 +15771,17 @@
         <v>3.99</v>
       </c>
     </row>
+    <row r="130" spans="1:3" ht="16" customHeight="1">
+      <c r="A130" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B130" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C130" s="3">
+        <v>3.58</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -15677,7 +15790,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C129"/>
+  <dimension ref="A1:C130"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -17104,6 +17217,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="130" spans="1:3" ht="16" customHeight="1">
+      <c r="A130" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B130" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C130" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -17112,7 +17236,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C129"/>
+  <dimension ref="A1:C130"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -18539,6 +18663,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="130" spans="1:3" ht="16" customHeight="1">
+      <c r="A130" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B130" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C130" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-17 13:59:02
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3563" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3584" uniqueCount="134">
   <si>
     <t>Date</t>
   </si>
@@ -425,6 +425,9 @@
   <si>
     <t>2026-10-16</t>
   </si>
+  <si>
+    <t>2026-10-17</t>
+  </si>
 </sst>
 </file>
 
@@ -540,7 +543,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -560,7 +563,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1330,7 +1333,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C130"/>
+  <dimension ref="A1:C131"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2768,6 +2771,17 @@
         <v>8.99</v>
       </c>
     </row>
+    <row r="131" spans="1:3" ht="16" customHeight="1">
+      <c r="A131" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B131" s="3">
+        <v>10.08</v>
+      </c>
+      <c r="C131" s="3">
+        <v>8.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2776,7 +2790,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C130"/>
+  <dimension ref="A1:C131"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4214,6 +4228,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="131" spans="1:3" ht="16" customHeight="1">
+      <c r="A131" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B131" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C131" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4222,7 +4247,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C130"/>
+  <dimension ref="A1:C131"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5660,6 +5685,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="131" spans="1:3" ht="16" customHeight="1">
+      <c r="A131" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B131" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C131" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5668,7 +5704,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C130"/>
+  <dimension ref="A1:C131"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7106,6 +7142,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="131" spans="1:3" ht="16" customHeight="1">
+      <c r="A131" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B131" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C131" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7114,7 +7161,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C130"/>
+  <dimension ref="A1:C131"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8552,6 +8599,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="131" spans="1:3" ht="16" customHeight="1">
+      <c r="A131" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B131" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C131" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8560,7 +8618,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C130"/>
+  <dimension ref="A1:C131"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9998,6 +10056,17 @@
         <v>7.99</v>
       </c>
     </row>
+    <row r="131" spans="1:3" ht="16" customHeight="1">
+      <c r="A131" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B131" s="3">
+        <v>8.1488</v>
+      </c>
+      <c r="C131" s="3">
+        <v>7.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10006,7 +10075,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C130"/>
+  <dimension ref="A1:C131"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11444,6 +11513,17 @@
         <v>3.79</v>
       </c>
     </row>
+    <row r="131" spans="1:3" ht="16" customHeight="1">
+      <c r="A131" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B131" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C131" s="3">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11452,7 +11532,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C130"/>
+  <dimension ref="A1:C131"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12890,6 +12970,17 @@
         <v>5.29</v>
       </c>
     </row>
+    <row r="131" spans="1:3" ht="16" customHeight="1">
+      <c r="A131" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B131" s="3">
+        <v>5.545</v>
+      </c>
+      <c r="C131" s="3">
+        <v>5.29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12898,7 +12989,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C130"/>
+  <dimension ref="A1:C131"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14336,6 +14427,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="131" spans="1:3" ht="16" customHeight="1">
+      <c r="A131" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B131" s="3">
+        <v>1.99</v>
+      </c>
+      <c r="C131" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14344,7 +14446,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C130"/>
+  <dimension ref="A1:C131"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15782,6 +15884,17 @@
         <v>3.58</v>
       </c>
     </row>
+    <row r="131" spans="1:3" ht="16" customHeight="1">
+      <c r="A131" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B131" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C131" s="3">
+        <v>3.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -15790,7 +15903,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C130"/>
+  <dimension ref="A1:C131"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -17228,6 +17341,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="131" spans="1:3" ht="16" customHeight="1">
+      <c r="A131" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B131" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C131" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -17236,7 +17360,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C130"/>
+  <dimension ref="A1:C131"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -18674,6 +18798,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="131" spans="1:3" ht="16" customHeight="1">
+      <c r="A131" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B131" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C131" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-18 14:11:25
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3584" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3607" uniqueCount="135">
   <si>
     <t>Date</t>
   </si>
@@ -427,6 +427,9 @@
   </si>
   <si>
     <t>2026-10-17</t>
+  </si>
+  <si>
+    <t>2026-10-18</t>
   </si>
 </sst>
 </file>
@@ -1333,7 +1336,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C131"/>
+  <dimension ref="A1:C132"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2782,6 +2785,17 @@
         <v>8.99</v>
       </c>
     </row>
+    <row r="132" spans="1:3" ht="16" customHeight="1">
+      <c r="A132" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B132" s="3">
+        <v>10.18</v>
+      </c>
+      <c r="C132" s="3">
+        <v>8.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2790,7 +2804,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C131"/>
+  <dimension ref="A1:C132"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4239,6 +4253,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="132" spans="1:3" ht="16" customHeight="1">
+      <c r="A132" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B132" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C132" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4247,7 +4272,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C131"/>
+  <dimension ref="A1:C132"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5696,6 +5721,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="132" spans="1:3" ht="16" customHeight="1">
+      <c r="A132" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B132" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C132" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5704,7 +5740,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C131"/>
+  <dimension ref="A1:C132"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7153,6 +7189,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="132" spans="1:3" ht="16" customHeight="1">
+      <c r="A132" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B132" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C132" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7161,7 +7208,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C131"/>
+  <dimension ref="A1:C132"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8610,6 +8657,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="132" spans="1:3" ht="16" customHeight="1">
+      <c r="A132" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B132" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C132" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8618,7 +8676,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C131"/>
+  <dimension ref="A1:C132"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10067,6 +10125,17 @@
         <v>7.99</v>
       </c>
     </row>
+    <row r="132" spans="1:3" ht="16" customHeight="1">
+      <c r="A132" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B132" s="3">
+        <v>8.029</v>
+      </c>
+      <c r="C132" s="3">
+        <v>7.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10075,7 +10144,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C131"/>
+  <dimension ref="A1:C132"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11524,6 +11593,17 @@
         <v>8</v>
       </c>
     </row>
+    <row r="132" spans="1:3" ht="16" customHeight="1">
+      <c r="A132" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B132" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C132" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11532,7 +11612,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C131"/>
+  <dimension ref="A1:C132"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12981,6 +13061,17 @@
         <v>5.29</v>
       </c>
     </row>
+    <row r="132" spans="1:3" ht="16" customHeight="1">
+      <c r="A132" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B132" s="3">
+        <v>5.6</v>
+      </c>
+      <c r="C132" s="3">
+        <v>5.29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12989,7 +13080,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C131"/>
+  <dimension ref="A1:C132"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14438,6 +14529,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="132" spans="1:3" ht="16" customHeight="1">
+      <c r="A132" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B132" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C132" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14446,7 +14548,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C131"/>
+  <dimension ref="A1:C132"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15895,6 +15997,17 @@
         <v>3.5</v>
       </c>
     </row>
+    <row r="132" spans="1:3" ht="16" customHeight="1">
+      <c r="A132" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B132" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C132" s="3">
+        <v>3.74</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -15903,7 +16016,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C131"/>
+  <dimension ref="A1:C132"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -17352,6 +17465,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="132" spans="1:3" ht="16" customHeight="1">
+      <c r="A132" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B132" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C132" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -17360,7 +17484,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C131"/>
+  <dimension ref="A1:C132"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -18809,6 +18933,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="132" spans="1:3" ht="16" customHeight="1">
+      <c r="A132" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B132" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C132" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-19 17:13:52
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3607" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3632" uniqueCount="136">
   <si>
     <t>Date</t>
   </si>
@@ -430,6 +430,9 @@
   </si>
   <si>
     <t>2026-10-18</t>
+  </si>
+  <si>
+    <t>2026-10-19</t>
   </si>
 </sst>
 </file>
@@ -1336,7 +1339,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C132"/>
+  <dimension ref="A1:C133"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2796,6 +2799,17 @@
         <v>8.99</v>
       </c>
     </row>
+    <row r="133" spans="1:3" ht="16" customHeight="1">
+      <c r="A133" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B133" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C133" s="3">
+        <v>8.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2804,7 +2818,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C132"/>
+  <dimension ref="A1:C133"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4264,6 +4278,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="133" spans="1:3" ht="16" customHeight="1">
+      <c r="A133" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B133" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C133" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4272,7 +4297,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C132"/>
+  <dimension ref="A1:C133"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5732,6 +5757,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="133" spans="1:3" ht="16" customHeight="1">
+      <c r="A133" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B133" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C133" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5740,7 +5776,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C132"/>
+  <dimension ref="A1:C133"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7200,6 +7236,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="133" spans="1:3" ht="16" customHeight="1">
+      <c r="A133" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B133" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C133" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7208,7 +7255,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C132"/>
+  <dimension ref="A1:C133"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8668,6 +8715,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="133" spans="1:3" ht="16" customHeight="1">
+      <c r="A133" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B133" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C133" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8676,7 +8734,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C132"/>
+  <dimension ref="A1:C133"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10136,6 +10194,17 @@
         <v>7.99</v>
       </c>
     </row>
+    <row r="133" spans="1:3" ht="16" customHeight="1">
+      <c r="A133" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B133" s="3">
+        <v>8.789999999999999</v>
+      </c>
+      <c r="C133" s="3">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10144,7 +10213,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C132"/>
+  <dimension ref="A1:C133"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11604,6 +11673,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="133" spans="1:3" ht="16" customHeight="1">
+      <c r="A133" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B133" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C133" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11612,7 +11692,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C132"/>
+  <dimension ref="A1:C133"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13072,6 +13152,17 @@
         <v>5.29</v>
       </c>
     </row>
+    <row r="133" spans="1:3" ht="16" customHeight="1">
+      <c r="A133" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B133" s="3">
+        <v>5.658</v>
+      </c>
+      <c r="C133" s="3">
+        <v>5.29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13080,7 +13171,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C132"/>
+  <dimension ref="A1:C133"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14540,6 +14631,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="133" spans="1:3" ht="16" customHeight="1">
+      <c r="A133" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B133" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C133" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14548,7 +14650,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C132"/>
+  <dimension ref="A1:C133"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -16008,6 +16110,17 @@
         <v>3.74</v>
       </c>
     </row>
+    <row r="133" spans="1:3" ht="16" customHeight="1">
+      <c r="A133" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B133" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C133" s="3">
+        <v>3.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -16016,7 +16129,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C132"/>
+  <dimension ref="A1:C133"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -17476,6 +17589,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="133" spans="1:3" ht="16" customHeight="1">
+      <c r="A133" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B133" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C133" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -17484,7 +17608,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C132"/>
+  <dimension ref="A1:C133"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -18944,6 +19068,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="133" spans="1:3" ht="16" customHeight="1">
+      <c r="A133" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B133" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C133" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-20 15:25:01
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3632" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3654" uniqueCount="137">
   <si>
     <t>Date</t>
   </si>
@@ -433,6 +433,9 @@
   </si>
   <si>
     <t>2026-10-19</t>
+  </si>
+  <si>
+    <t>2026-10-20</t>
   </si>
 </sst>
 </file>
@@ -1339,7 +1342,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C133"/>
+  <dimension ref="A1:C134"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2810,6 +2813,17 @@
         <v>8.99</v>
       </c>
     </row>
+    <row r="134" spans="1:3" ht="16" customHeight="1">
+      <c r="A134" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B134" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C134" s="3">
+        <v>8.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2818,7 +2832,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C133"/>
+  <dimension ref="A1:C134"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4289,6 +4303,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="134" spans="1:3" ht="16" customHeight="1">
+      <c r="A134" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B134" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C134" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4297,7 +4322,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C133"/>
+  <dimension ref="A1:C134"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5768,6 +5793,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="134" spans="1:3" ht="16" customHeight="1">
+      <c r="A134" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B134" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C134" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5776,7 +5812,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C133"/>
+  <dimension ref="A1:C134"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7247,6 +7283,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="134" spans="1:3" ht="16" customHeight="1">
+      <c r="A134" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B134" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C134" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7255,7 +7302,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C133"/>
+  <dimension ref="A1:C134"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8726,6 +8773,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="134" spans="1:3" ht="16" customHeight="1">
+      <c r="A134" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B134" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C134" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8734,7 +8792,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C133"/>
+  <dimension ref="A1:C134"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10205,6 +10263,17 @@
         <v>9</v>
       </c>
     </row>
+    <row r="134" spans="1:3" ht="16" customHeight="1">
+      <c r="A134" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B134" s="3">
+        <v>6</v>
+      </c>
+      <c r="C134" s="3">
+        <v>7.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10213,7 +10282,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C133"/>
+  <dimension ref="A1:C134"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11684,6 +11753,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="134" spans="1:3" ht="16" customHeight="1">
+      <c r="A134" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B134" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C134" s="3">
+        <v>3.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11692,7 +11772,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C133"/>
+  <dimension ref="A1:C134"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13163,6 +13243,17 @@
         <v>5.29</v>
       </c>
     </row>
+    <row r="134" spans="1:3" ht="16" customHeight="1">
+      <c r="A134" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B134" s="3">
+        <v>5.715</v>
+      </c>
+      <c r="C134" s="3">
+        <v>5.29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13171,7 +13262,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C133"/>
+  <dimension ref="A1:C134"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14642,6 +14733,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="134" spans="1:3" ht="16" customHeight="1">
+      <c r="A134" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B134" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C134" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14650,7 +14752,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C133"/>
+  <dimension ref="A1:C134"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -16121,6 +16223,17 @@
         <v>3.99</v>
       </c>
     </row>
+    <row r="134" spans="1:3" ht="16" customHeight="1">
+      <c r="A134" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B134" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C134" s="3">
+        <v>3.58</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -16129,7 +16242,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C133"/>
+  <dimension ref="A1:C134"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -17600,6 +17713,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="134" spans="1:3" ht="16" customHeight="1">
+      <c r="A134" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B134" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C134" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -17608,7 +17732,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C133"/>
+  <dimension ref="A1:C134"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -19079,6 +19203,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="134" spans="1:3" ht="16" customHeight="1">
+      <c r="A134" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B134" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C134" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-21 15:41:45
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3654" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3678" uniqueCount="138">
   <si>
     <t>Date</t>
   </si>
@@ -436,6 +436,9 @@
   </si>
   <si>
     <t>2026-10-20</t>
+  </si>
+  <si>
+    <t>2026-10-21</t>
   </si>
 </sst>
 </file>
@@ -1342,7 +1345,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C134"/>
+  <dimension ref="A1:C135"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2824,6 +2827,17 @@
         <v>8.99</v>
       </c>
     </row>
+    <row r="135" spans="1:3" ht="16" customHeight="1">
+      <c r="A135" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B135" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C135" s="3">
+        <v>8.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2832,7 +2846,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C134"/>
+  <dimension ref="A1:C135"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4314,6 +4328,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="135" spans="1:3" ht="16" customHeight="1">
+      <c r="A135" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B135" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C135" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4322,7 +4347,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C134"/>
+  <dimension ref="A1:C135"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5804,6 +5829,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="135" spans="1:3" ht="16" customHeight="1">
+      <c r="A135" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B135" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C135" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5812,7 +5848,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C134"/>
+  <dimension ref="A1:C135"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7294,6 +7330,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="135" spans="1:3" ht="16" customHeight="1">
+      <c r="A135" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B135" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C135" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7302,7 +7349,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C134"/>
+  <dimension ref="A1:C135"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8784,6 +8831,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="135" spans="1:3" ht="16" customHeight="1">
+      <c r="A135" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B135" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C135" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8792,7 +8850,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C134"/>
+  <dimension ref="A1:C135"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10274,6 +10332,17 @@
         <v>7.99</v>
       </c>
     </row>
+    <row r="135" spans="1:3" ht="16" customHeight="1">
+      <c r="A135" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B135" s="3">
+        <v>8.789999999999999</v>
+      </c>
+      <c r="C135" s="3">
+        <v>7.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10282,7 +10351,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C134"/>
+  <dimension ref="A1:C135"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11764,6 +11833,17 @@
         <v>3.79</v>
       </c>
     </row>
+    <row r="135" spans="1:3" ht="16" customHeight="1">
+      <c r="A135" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B135" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C135" s="3">
+        <v>3.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11772,7 +11852,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C134"/>
+  <dimension ref="A1:C135"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13254,6 +13334,17 @@
         <v>5.29</v>
       </c>
     </row>
+    <row r="135" spans="1:3" ht="16" customHeight="1">
+      <c r="A135" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B135" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C135" s="3">
+        <v>5.29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13262,7 +13353,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C134"/>
+  <dimension ref="A1:C135"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14744,6 +14835,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="135" spans="1:3" ht="16" customHeight="1">
+      <c r="A135" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B135" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C135" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14752,7 +14854,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C134"/>
+  <dimension ref="A1:C135"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -16234,6 +16336,17 @@
         <v>3.58</v>
       </c>
     </row>
+    <row r="135" spans="1:3" ht="16" customHeight="1">
+      <c r="A135" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B135" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C135" s="3">
+        <v>3.22</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -16242,7 +16355,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C134"/>
+  <dimension ref="A1:C135"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -17724,6 +17837,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="135" spans="1:3" ht="16" customHeight="1">
+      <c r="A135" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B135" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C135" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -17732,7 +17856,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C134"/>
+  <dimension ref="A1:C135"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -19214,6 +19338,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="135" spans="1:3" ht="16" customHeight="1">
+      <c r="A135" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B135" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C135" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-23 15:30:05
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3701" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3723" uniqueCount="140">
   <si>
     <t>Date</t>
   </si>
@@ -443,6 +443,9 @@
   <si>
     <t>2026-10-22</t>
   </si>
+  <si>
+    <t>2026-10-23</t>
+  </si>
 </sst>
 </file>
 
@@ -558,13 +561,56 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
+      <xdr:colOff>65821</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>139013</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="NVIDIA_B300_SXM6.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3952875" y="0"/>
+          <a:ext cx="7990621" cy="4368113"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
       <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1" descr="NVIDIA_B300_SXM6.png"/>
+        <xdr:cNvPr id="2" name="Picture 1" descr="AMD_Instinct_MI300X.png"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -590,49 +636,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>139013</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1" descr="AMD_Instinct_MI300X.png"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
 <file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
@@ -644,7 +647,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -664,7 +667,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -687,7 +690,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -707,7 +710,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -773,56 +776,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Picture 1" descr="NVIDIA_B200_SXM.png"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>139013</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1" descr="NVIDIA_H200_NVL.png"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -848,6 +808,49 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>65821</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>139013</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="NVIDIA_H200_NVL.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3952875" y="0"/>
+          <a:ext cx="7990621" cy="4368113"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
@@ -859,7 +862,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -879,7 +882,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -902,7 +905,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -922,7 +925,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -945,7 +948,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -965,7 +968,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -988,7 +991,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -1008,7 +1011,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1348,7 +1351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C136"/>
+  <dimension ref="A1:C137"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2852,6 +2855,17 @@
         <v>8.99</v>
       </c>
     </row>
+    <row r="137" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A137" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B137" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C137" s="3">
+        <v>8.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2860,7 +2874,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C136"/>
+  <dimension ref="A1:C137"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4364,6 +4378,17 @@
         <v>2.39</v>
       </c>
     </row>
+    <row r="137" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A137" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B137" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C137" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4372,7 +4397,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C136"/>
+  <dimension ref="A1:C137"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5876,6 +5901,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="137" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A137" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B137" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C137" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5884,7 +5920,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C136"/>
+  <dimension ref="A1:C137"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7388,6 +7424,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="137" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A137" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B137" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C137" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7396,7 +7443,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C136"/>
+  <dimension ref="A1:C137"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8900,6 +8947,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="137" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A137" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B137" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C137" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8908,7 +8966,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C136"/>
+  <dimension ref="A1:C137"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10412,6 +10470,17 @@
         <v>7.99</v>
       </c>
     </row>
+    <row r="137" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A137" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B137" s="3">
+        <v>8.355</v>
+      </c>
+      <c r="C137" s="3">
+        <v>7.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10420,7 +10489,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C136"/>
+  <dimension ref="A1:C137"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11924,6 +11993,17 @@
         <v>3.79</v>
       </c>
     </row>
+    <row r="137" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A137" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B137" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C137" s="3">
+        <v>5.5333</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11932,7 +12012,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C136"/>
+  <dimension ref="A1:C137"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13436,6 +13516,17 @@
         <v>5.29</v>
       </c>
     </row>
+    <row r="137" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A137" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B137" s="3">
+        <v>5.89</v>
+      </c>
+      <c r="C137" s="3">
+        <v>5.29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13444,7 +13535,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C136"/>
+  <dimension ref="A1:C137"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14948,6 +15039,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="137" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A137" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B137" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C137" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14956,7 +15058,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C136"/>
+  <dimension ref="A1:C137"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -16460,6 +16562,17 @@
         <v>3.904</v>
       </c>
     </row>
+    <row r="137" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A137" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B137" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C137" s="3">
+        <v>3.9867</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -16468,7 +16581,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C136"/>
+  <dimension ref="A1:C137"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -17972,6 +18085,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="137" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A137" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B137" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C137" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -17980,7 +18104,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C136"/>
+  <dimension ref="A1:C137"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -19484,6 +19608,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="137" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A137" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B137" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C137" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-24 14:09:04
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3723" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3746" uniqueCount="141">
   <si>
     <t>Date</t>
   </si>
@@ -446,6 +446,9 @@
   <si>
     <t>2026-10-23</t>
   </si>
+  <si>
+    <t>2026-10-24</t>
+  </si>
 </sst>
 </file>
 
@@ -604,7 +607,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>65821</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -624,7 +627,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="7990621" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -647,7 +650,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>65821</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -667,7 +670,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="7990621" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -690,7 +693,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>65821</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -710,7 +713,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="7990621" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -776,7 +779,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>65821</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -796,7 +799,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="7990621" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -862,7 +865,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>65821</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -882,7 +885,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="7990621" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -905,7 +908,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>65821</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -925,7 +928,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="7990621" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -948,7 +951,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>65821</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -968,7 +971,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="7990621" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -991,7 +994,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>65821</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -1011,7 +1014,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="7990621" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1351,7 +1354,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C137"/>
+  <dimension ref="A1:C138"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2866,6 +2869,17 @@
         <v>8.99</v>
       </c>
     </row>
+    <row r="138" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A138" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B138" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C138" s="3">
+        <v>8.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2874,7 +2888,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C137"/>
+  <dimension ref="A1:C138"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4389,6 +4403,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="138" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A138" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B138" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C138" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4397,7 +4422,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C137"/>
+  <dimension ref="A1:C138"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5912,6 +5937,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="138" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A138" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B138" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C138" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5920,7 +5956,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C137"/>
+  <dimension ref="A1:C138"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7435,6 +7471,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="138" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A138" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B138" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C138" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7443,7 +7490,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C137"/>
+  <dimension ref="A1:C138"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8958,6 +9005,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="138" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A138" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B138" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C138" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8966,7 +9024,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C137"/>
+  <dimension ref="A1:C138"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10481,6 +10539,17 @@
         <v>7.99</v>
       </c>
     </row>
+    <row r="138" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A138" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B138" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C138" s="3">
+        <v>7.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10489,7 +10558,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C137"/>
+  <dimension ref="A1:C138"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12004,6 +12073,17 @@
         <v>5.5333</v>
       </c>
     </row>
+    <row r="138" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A138" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B138" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C138" s="3">
+        <v>4.6867</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12012,7 +12092,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C137"/>
+  <dimension ref="A1:C138"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13527,6 +13607,17 @@
         <v>5.29</v>
       </c>
     </row>
+    <row r="138" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A138" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B138" s="3">
+        <v>5.9475</v>
+      </c>
+      <c r="C138" s="3">
+        <v>5.29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13535,7 +13626,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C137"/>
+  <dimension ref="A1:C138"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15050,6 +15141,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="138" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A138" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B138" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C138" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -15058,7 +15160,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C137"/>
+  <dimension ref="A1:C138"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -16573,6 +16675,17 @@
         <v>3.9867</v>
       </c>
     </row>
+    <row r="138" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A138" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B138" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C138" s="3">
+        <v>3.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -16581,7 +16694,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C137"/>
+  <dimension ref="A1:C138"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -18096,6 +18209,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="138" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A138" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B138" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C138" s="3">
+        <v>3.66</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -18104,7 +18228,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C137"/>
+  <dimension ref="A1:C138"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -19619,6 +19743,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="138" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A138" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B138" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C138" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-25 14:37:15
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3746" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3769" uniqueCount="142">
   <si>
     <t>Date</t>
   </si>
@@ -449,6 +449,9 @@
   <si>
     <t>2026-10-24</t>
   </si>
+  <si>
+    <t>2026-10-25</t>
+  </si>
 </sst>
 </file>
 
@@ -564,7 +567,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>65821</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -584,7 +587,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7990621" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -607,7 +610,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>65821</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -627,7 +630,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7990621" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -650,7 +653,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>65821</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -670,7 +673,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7990621" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -693,7 +696,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>65821</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -713,7 +716,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7990621" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -779,7 +782,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>65821</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -799,7 +802,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7990621" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -822,7 +825,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>65821</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -842,7 +845,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7990621" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -865,7 +868,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>65821</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -885,7 +888,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7990621" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -908,7 +911,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>65821</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -928,7 +931,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7990621" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -951,7 +954,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>65821</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -971,7 +974,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7990621" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -994,7 +997,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>65821</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -1014,7 +1017,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7990621" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1354,7 +1357,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C138"/>
+  <dimension ref="A1:C139"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2880,6 +2883,17 @@
         <v>8.99</v>
       </c>
     </row>
+    <row r="139" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A139" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B139" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C139" s="3">
+        <v>8.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2888,7 +2902,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C138"/>
+  <dimension ref="A1:C139"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4414,6 +4428,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="139" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A139" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B139" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C139" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4422,7 +4447,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C138"/>
+  <dimension ref="A1:C139"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5948,6 +5973,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="139" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A139" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B139" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C139" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5956,7 +5992,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C138"/>
+  <dimension ref="A1:C139"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7482,6 +7518,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="139" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A139" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B139" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C139" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7490,7 +7537,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C138"/>
+  <dimension ref="A1:C139"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9016,6 +9063,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="139" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A139" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B139" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C139" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9024,7 +9082,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C138"/>
+  <dimension ref="A1:C139"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10550,6 +10608,17 @@
         <v>7.99</v>
       </c>
     </row>
+    <row r="139" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A139" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B139" s="3">
+        <v>8.789999999999999</v>
+      </c>
+      <c r="C139" s="3">
+        <v>7.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10558,7 +10627,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C138"/>
+  <dimension ref="A1:C139"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12084,6 +12153,17 @@
         <v>4.6867</v>
       </c>
     </row>
+    <row r="139" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A139" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B139" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C139" s="3">
+        <v>3.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12092,7 +12172,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C138"/>
+  <dimension ref="A1:C139"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13618,6 +13698,17 @@
         <v>5.29</v>
       </c>
     </row>
+    <row r="139" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A139" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B139" s="3">
+        <v>5.945</v>
+      </c>
+      <c r="C139" s="3">
+        <v>5.29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13626,7 +13717,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C138"/>
+  <dimension ref="A1:C139"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15152,6 +15243,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="139" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A139" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B139" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C139" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -15160,7 +15262,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C138"/>
+  <dimension ref="A1:C139"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -16686,6 +16788,17 @@
         <v>3.99</v>
       </c>
     </row>
+    <row r="139" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A139" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B139" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C139" s="3">
+        <v>3.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -16694,7 +16807,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C138"/>
+  <dimension ref="A1:C139"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -18220,6 +18333,17 @@
         <v>3.66</v>
       </c>
     </row>
+    <row r="139" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A139" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B139" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C139" s="3">
+        <v>3.9867</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -18228,7 +18352,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C138"/>
+  <dimension ref="A1:C139"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -19754,6 +19878,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="139" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A139" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B139" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C139" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-26 17:02:27
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3769" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3793" uniqueCount="143">
   <si>
     <t>Date</t>
   </si>
@@ -451,6 +451,9 @@
   </si>
   <si>
     <t>2026-10-25</t>
+  </si>
+  <si>
+    <t>2026-10-26</t>
   </si>
 </sst>
 </file>
@@ -1357,7 +1360,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C139"/>
+  <dimension ref="A1:C140"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2894,6 +2897,17 @@
         <v>8.99</v>
       </c>
     </row>
+    <row r="140" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A140" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B140" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C140" s="3">
+        <v>8.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2902,7 +2916,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C139"/>
+  <dimension ref="A1:C140"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4439,6 +4453,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="140" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A140" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B140" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C140" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4447,7 +4472,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C139"/>
+  <dimension ref="A1:C140"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5984,6 +6009,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="140" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A140" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B140" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C140" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5992,7 +6028,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C139"/>
+  <dimension ref="A1:C140"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7529,6 +7565,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="140" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A140" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B140" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C140" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7537,7 +7584,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C139"/>
+  <dimension ref="A1:C140"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9074,6 +9121,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="140" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A140" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B140" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C140" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9082,7 +9140,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C139"/>
+  <dimension ref="A1:C140"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10619,6 +10677,17 @@
         <v>7.99</v>
       </c>
     </row>
+    <row r="140" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A140" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B140" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C140" s="3">
+        <v>7.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10627,7 +10696,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C139"/>
+  <dimension ref="A1:C140"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12164,6 +12233,17 @@
         <v>3.79</v>
       </c>
     </row>
+    <row r="140" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A140" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B140" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C140" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12172,7 +12252,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C139"/>
+  <dimension ref="A1:C140"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13709,6 +13789,17 @@
         <v>5.29</v>
       </c>
     </row>
+    <row r="140" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A140" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B140" s="3">
+        <v>6.005</v>
+      </c>
+      <c r="C140" s="3">
+        <v>5.29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13717,7 +13808,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C139"/>
+  <dimension ref="A1:C140"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15254,6 +15345,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="140" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A140" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B140" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C140" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -15262,7 +15364,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C139"/>
+  <dimension ref="A1:C140"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -16799,6 +16901,17 @@
         <v>3.5</v>
       </c>
     </row>
+    <row r="140" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A140" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B140" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C140" s="3">
+        <v>2.2667</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -16807,7 +16920,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C139"/>
+  <dimension ref="A1:C140"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -18344,6 +18457,17 @@
         <v>3.9867</v>
       </c>
     </row>
+    <row r="140" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A140" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B140" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C140" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -18352,7 +18476,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C139"/>
+  <dimension ref="A1:C140"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -19889,6 +20013,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="140" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A140" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B140" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C140" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-27 16:05:16
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3793" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3817" uniqueCount="144">
   <si>
     <t>Date</t>
   </si>
@@ -454,6 +454,9 @@
   </si>
   <si>
     <t>2026-10-26</t>
+  </si>
+  <si>
+    <t>2026-10-27</t>
   </si>
 </sst>
 </file>
@@ -1360,7 +1363,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C140"/>
+  <dimension ref="A1:C141"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2908,6 +2911,17 @@
         <v>8.99</v>
       </c>
     </row>
+    <row r="141" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A141" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B141" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C141" s="3">
+        <v>8.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2916,7 +2930,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C140"/>
+  <dimension ref="A1:C141"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4464,6 +4478,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="141" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A141" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B141" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C141" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4472,7 +4497,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C140"/>
+  <dimension ref="A1:C141"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6020,6 +6045,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="141" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A141" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B141" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C141" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6028,7 +6064,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C140"/>
+  <dimension ref="A1:C141"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7576,6 +7612,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="141" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A141" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B141" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C141" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7584,7 +7631,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C140"/>
+  <dimension ref="A1:C141"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9132,6 +9179,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="141" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A141" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B141" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C141" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9140,7 +9198,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C140"/>
+  <dimension ref="A1:C141"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10688,6 +10746,17 @@
         <v>7.99</v>
       </c>
     </row>
+    <row r="141" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A141" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B141" s="3">
+        <v>8.789999999999999</v>
+      </c>
+      <c r="C141" s="3">
+        <v>7.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10696,7 +10765,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C140"/>
+  <dimension ref="A1:C141"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12244,6 +12313,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="141" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A141" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B141" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C141" s="3">
+        <v>3.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12252,7 +12332,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C140"/>
+  <dimension ref="A1:C141"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13800,6 +13880,17 @@
         <v>5.29</v>
       </c>
     </row>
+    <row r="141" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A141" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B141" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C141" s="3">
+        <v>5.29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13808,7 +13899,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C140"/>
+  <dimension ref="A1:C141"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15356,6 +15447,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="141" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A141" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B141" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C141" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -15364,7 +15466,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C140"/>
+  <dimension ref="A1:C141"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -16912,6 +17014,17 @@
         <v>2.2667</v>
       </c>
     </row>
+    <row r="141" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A141" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B141" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C141" s="3">
+        <v>3.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -16920,7 +17033,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C140"/>
+  <dimension ref="A1:C141"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -18468,6 +18581,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="141" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A141" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B141" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C141" s="3">
+        <v>3.9867</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -18476,7 +18600,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C140"/>
+  <dimension ref="A1:C141"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -20024,6 +20148,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="141" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A141" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B141" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C141" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-28 16:51:36
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3817" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3843" uniqueCount="145">
   <si>
     <t>Date</t>
   </si>
@@ -457,6 +457,9 @@
   </si>
   <si>
     <t>2026-10-27</t>
+  </si>
+  <si>
+    <t>2026-10-28</t>
   </si>
 </sst>
 </file>
@@ -1363,7 +1366,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C141"/>
+  <dimension ref="A1:C142"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2922,6 +2925,17 @@
         <v>8.99</v>
       </c>
     </row>
+    <row r="142" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A142" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B142" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C142" s="3">
+        <v>8.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2930,7 +2944,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C141"/>
+  <dimension ref="A1:C142"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4489,6 +4503,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="142" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A142" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B142" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C142" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4497,7 +4522,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C141"/>
+  <dimension ref="A1:C142"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6056,6 +6081,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="142" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A142" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B142" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C142" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6064,7 +6100,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C141"/>
+  <dimension ref="A1:C142"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7623,6 +7659,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="142" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A142" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B142" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C142" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7631,7 +7678,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C141"/>
+  <dimension ref="A1:C142"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9190,6 +9237,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="142" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A142" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B142" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C142" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9198,7 +9256,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C141"/>
+  <dimension ref="A1:C142"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10757,6 +10815,17 @@
         <v>7.99</v>
       </c>
     </row>
+    <row r="142" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A142" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B142" s="3">
+        <v>8.789999999999999</v>
+      </c>
+      <c r="C142" s="3">
+        <v>7.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10765,7 +10834,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C141"/>
+  <dimension ref="A1:C142"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12324,6 +12393,17 @@
         <v>3.79</v>
       </c>
     </row>
+    <row r="142" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A142" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B142" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C142" s="3">
+        <v>6.5333</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12332,7 +12412,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C141"/>
+  <dimension ref="A1:C142"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13891,6 +13971,17 @@
         <v>5.29</v>
       </c>
     </row>
+    <row r="142" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A142" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B142" s="3">
+        <v>6.1275</v>
+      </c>
+      <c r="C142" s="3">
+        <v>5.29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13899,7 +13990,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C141"/>
+  <dimension ref="A1:C142"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15458,6 +15549,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="142" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A142" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B142" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C142" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -15466,7 +15568,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C141"/>
+  <dimension ref="A1:C142"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -17025,6 +17127,17 @@
         <v>3.99</v>
       </c>
     </row>
+    <row r="142" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A142" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B142" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C142" s="3">
+        <v>3.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -17033,7 +17146,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C141"/>
+  <dimension ref="A1:C142"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -18592,6 +18705,17 @@
         <v>3.9867</v>
       </c>
     </row>
+    <row r="142" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A142" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B142" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C142" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -18600,7 +18724,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C141"/>
+  <dimension ref="A1:C142"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -20159,6 +20283,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="142" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A142" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B142" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C142" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-29 17:07:42
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3843" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3867" uniqueCount="146">
   <si>
     <t>Date</t>
   </si>
@@ -460,6 +460,9 @@
   </si>
   <si>
     <t>2026-10-28</t>
+  </si>
+  <si>
+    <t>2026-10-29</t>
   </si>
 </sst>
 </file>
@@ -1366,7 +1369,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C142"/>
+  <dimension ref="A1:C143"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2936,6 +2939,17 @@
         <v>8.99</v>
       </c>
     </row>
+    <row r="143" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A143" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B143" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C143" s="3">
+        <v>8.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2944,7 +2958,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C142"/>
+  <dimension ref="A1:C143"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4514,6 +4528,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="143" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A143" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B143" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C143" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4522,7 +4547,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C142"/>
+  <dimension ref="A1:C143"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6092,6 +6117,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="143" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A143" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B143" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C143" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6100,7 +6136,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C142"/>
+  <dimension ref="A1:C143"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7670,6 +7706,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="143" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A143" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B143" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C143" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7678,7 +7725,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C142"/>
+  <dimension ref="A1:C143"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9248,6 +9295,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="143" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A143" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B143" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C143" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9256,7 +9314,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C142"/>
+  <dimension ref="A1:C143"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10826,6 +10884,17 @@
         <v>7.99</v>
       </c>
     </row>
+    <row r="143" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A143" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B143" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C143" s="3">
+        <v>7.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10834,7 +10903,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C142"/>
+  <dimension ref="A1:C143"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12404,6 +12473,17 @@
         <v>6.5333</v>
       </c>
     </row>
+    <row r="143" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A143" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B143" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C143" s="3">
+        <v>5.6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12412,7 +12492,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C142"/>
+  <dimension ref="A1:C143"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13982,6 +14062,17 @@
         <v>5.29</v>
       </c>
     </row>
+    <row r="143" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A143" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B143" s="3">
+        <v>6.1875</v>
+      </c>
+      <c r="C143" s="3">
+        <v>5.29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13990,7 +14081,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C142"/>
+  <dimension ref="A1:C143"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15560,6 +15651,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="143" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A143" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B143" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C143" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -15568,7 +15670,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C142"/>
+  <dimension ref="A1:C143"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -17138,6 +17240,17 @@
         <v>3.99</v>
       </c>
     </row>
+    <row r="143" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A143" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B143" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C143" s="3">
+        <v>3.8627</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -17146,7 +17259,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C142"/>
+  <dimension ref="A1:C143"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -18716,6 +18829,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="143" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A143" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B143" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C143" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -18724,7 +18848,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C142"/>
+  <dimension ref="A1:C143"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -20294,6 +20418,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="143" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A143" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B143" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C143" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-30 16:50:43
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3867" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3891" uniqueCount="147">
   <si>
     <t>Date</t>
   </si>
@@ -464,6 +464,9 @@
   <si>
     <t>2026-10-29</t>
   </si>
+  <si>
+    <t>2026-10-30</t>
+  </si>
 </sst>
 </file>
 
@@ -794,7 +797,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -814,7 +817,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1369,7 +1372,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C143"/>
+  <dimension ref="A1:C144"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2950,6 +2953,17 @@
         <v>8.99</v>
       </c>
     </row>
+    <row r="144" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A144" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B144" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C144" s="3">
+        <v>8.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2958,7 +2972,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C143"/>
+  <dimension ref="A1:C144"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4539,6 +4553,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="144" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A144" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B144" s="3">
+        <v>2.59</v>
+      </c>
+      <c r="C144" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4547,7 +4572,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C143"/>
+  <dimension ref="A1:C144"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6128,6 +6153,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="144" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A144" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B144" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C144" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6136,7 +6172,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C143"/>
+  <dimension ref="A1:C144"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7717,6 +7753,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="144" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A144" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B144" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C144" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7725,7 +7772,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C143"/>
+  <dimension ref="A1:C144"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9306,6 +9353,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="144" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A144" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B144" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C144" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9314,7 +9372,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C143"/>
+  <dimension ref="A1:C144"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10895,6 +10953,17 @@
         <v>7.99</v>
       </c>
     </row>
+    <row r="144" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A144" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B144" s="3">
+        <v>8.789999999999999</v>
+      </c>
+      <c r="C144" s="3">
+        <v>10.25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10903,7 +10972,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C143"/>
+  <dimension ref="A1:C144"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12484,6 +12553,17 @@
         <v>5.6</v>
       </c>
     </row>
+    <row r="144" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A144" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B144" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C144" s="3">
+        <v>4.7987</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12492,7 +12572,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C143"/>
+  <dimension ref="A1:C144"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14073,6 +14153,17 @@
         <v>5.29</v>
       </c>
     </row>
+    <row r="144" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A144" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B144" s="3">
+        <v>6.19</v>
+      </c>
+      <c r="C144" s="3">
+        <v>5.29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14081,7 +14172,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C143"/>
+  <dimension ref="A1:C144"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15662,6 +15753,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="144" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A144" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B144" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C144" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -15670,7 +15772,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C143"/>
+  <dimension ref="A1:C144"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -17251,6 +17353,17 @@
         <v>3.8627</v>
       </c>
     </row>
+    <row r="144" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A144" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B144" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C144" s="3">
+        <v>3.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -17259,7 +17372,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C143"/>
+  <dimension ref="A1:C144"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -18840,6 +18953,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="144" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A144" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B144" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C144" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -18848,7 +18972,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C143"/>
+  <dimension ref="A1:C144"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -20429,6 +20553,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="144" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A144" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B144" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C144" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-10-31 15:54:16
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3891" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3911" uniqueCount="148">
   <si>
     <t>Date</t>
   </si>
@@ -466,6 +466,9 @@
   </si>
   <si>
     <t>2026-10-30</t>
+  </si>
+  <si>
+    <t>2026-10-31</t>
   </si>
 </sst>
 </file>
@@ -1372,7 +1375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C144"/>
+  <dimension ref="A1:C145"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2964,6 +2967,17 @@
         <v>8.99</v>
       </c>
     </row>
+    <row r="145" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A145" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B145" s="3">
+        <v>11.09</v>
+      </c>
+      <c r="C145" s="3">
+        <v>8.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2972,7 +2986,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C144"/>
+  <dimension ref="A1:C145"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4564,6 +4578,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="145" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A145" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B145" s="3">
+        <v>2.59</v>
+      </c>
+      <c r="C145" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4572,7 +4597,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C144"/>
+  <dimension ref="A1:C145"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6164,6 +6189,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="145" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A145" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B145" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C145" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6172,7 +6208,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C144"/>
+  <dimension ref="A1:C145"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7764,6 +7800,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="145" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A145" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B145" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C145" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7772,7 +7819,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C144"/>
+  <dimension ref="A1:C145"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9364,6 +9411,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="145" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A145" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B145" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C145" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9372,7 +9430,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C144"/>
+  <dimension ref="A1:C145"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10964,6 +11022,17 @@
         <v>10.25</v>
       </c>
     </row>
+    <row r="145" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A145" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B145" s="3">
+        <v>8.789999999999999</v>
+      </c>
+      <c r="C145" s="3">
+        <v>7.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10972,7 +11041,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C144"/>
+  <dimension ref="A1:C145"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12564,6 +12633,17 @@
         <v>4.7987</v>
       </c>
     </row>
+    <row r="145" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A145" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B145" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C145" s="3">
+        <v>3.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12572,7 +12652,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C144"/>
+  <dimension ref="A1:C145"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14164,6 +14244,17 @@
         <v>5.29</v>
       </c>
     </row>
+    <row r="145" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A145" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B145" s="3">
+        <v>6.19</v>
+      </c>
+      <c r="C145" s="3">
+        <v>5.29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14172,7 +14263,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C144"/>
+  <dimension ref="A1:C145"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -15764,6 +15855,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="145" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A145" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B145" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C145" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -15772,7 +15874,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C144"/>
+  <dimension ref="A1:C145"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -17364,6 +17466,17 @@
         <v>3.99</v>
       </c>
     </row>
+    <row r="145" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A145" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B145" s="3">
+        <v>0</v>
+      </c>
+      <c r="C145" s="3">
+        <v>3.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -17372,7 +17485,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C144"/>
+  <dimension ref="A1:C145"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -18964,6 +19077,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="145" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A145" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B145" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C145" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -18972,7 +19096,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C144"/>
+  <dimension ref="A1:C145"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -20564,6 +20688,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="145" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A145" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B145" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C145" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>